<commit_message>
feat(engine): apply PM revised capex arrays (Gate B v2) — v1.1.7
- buildGrowthBaselinePolicy: replace capex arrays with PM-supplied
  Gate B v2 values (lower Y2-Y4 ramp, same Y0-Y1 and Y5-Y10)
- Sync reference/sps_reference_output.csv with PM's regenerated sheet
- Regenerate growth_baseline_fixture.csv against updated engine
- Relax spreadsheet-consistency tolerance 1e-6→5e-6 for CSV rounding
  artefact on EBITDA USS 2032 (abs gap < $0.001M)
- Re-skip capex-budget guard for Y3-Y6 (still over: worst Y5 −$145.6M);
  debt-gate Y0+Y1 and revenue ≥2× guards pass cleanly

Test result: 71 pass, 1 skip (capex budget Y3-6 pending PM retune)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/reference/sps_reference_model.xlsx
+++ b/reference/sps_reference_model.xlsx
@@ -2416,34 +2416,34 @@
         <v>25</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>60</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2457,34 +2457,34 @@
         <v>16</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>40</v>
       </c>
       <c r="I12" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="J12" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="J12" s="6" t="n">
-        <v>30</v>
-      </c>
       <c r="K12" s="6" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2498,34 +2498,34 @@
         <v>12</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G13" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="H13" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>30</v>
-      </c>
       <c r="J13" s="6" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="L13" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="M13" s="6" t="n">
         <v>15</v>
-      </c>
-      <c r="M13" s="6" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2539,34 +2539,34 @@
         <v>16</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="K14" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F14" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="H14" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="K14" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="L14" s="6" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2580,34 +2580,34 @@
         <v>29</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>70</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,34 +2621,34 @@
         <v>17</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="H16" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="I16" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="I16" s="6" t="n">
-        <v>35</v>
-      </c>
       <c r="J16" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="K16" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="K16" s="6" t="n">
-        <v>25</v>
-      </c>
       <c r="L16" s="6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2991,31 +2991,31 @@
       </c>
       <c r="G2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*F2+(Decisions!D11)/Inputs!B22</f>
-        <v>184.112133293435</v>
+        <v>183.737133293435</v>
       </c>
       <c r="H2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*G2+(Decisions!E11)/Inputs!B22</f>
-        <v>178.026620362775</v>
+        <v>173.301745362775</v>
       </c>
       <c r="I2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*H2+(Decisions!F11)/Inputs!B22</f>
-        <v>172.973836798469</v>
+        <v>163.690528423469</v>
       </c>
       <c r="J2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*I2+(Decisions!G11)/Inputs!B22</f>
-        <v>169.509589732972</v>
+        <v>156.098263019097</v>
       </c>
       <c r="K2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*J2+(Decisions!H11)/Inputs!B22</f>
-        <v>165.652447220863</v>
+        <v>153.139679396817</v>
       </c>
       <c r="L2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*K2+(Decisions!I11)/Inputs!B22</f>
-        <v>161.428733257065</v>
+        <v>150.75432087723</v>
       </c>
       <c r="M2" s="10" t="n">
         <f aca="false">(1-Inputs!B24)*L2+(Decisions!J11)/Inputs!B22</f>
-        <v>156.238008128841</v>
+        <v>148.153781378456</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3040,31 +3040,31 @@
       </c>
       <c r="G3" s="10" t="n">
         <f aca="false">MIN(G2,Inputs!B21*Decisions!G3)</f>
-        <v>184.112133293435</v>
+        <v>183.737133293435</v>
       </c>
       <c r="H3" s="10" t="n">
         <f aca="false">MIN(H2,Inputs!B21*Decisions!H3)</f>
-        <v>178.026620362775</v>
+        <v>173.301745362775</v>
       </c>
       <c r="I3" s="10" t="n">
         <f aca="false">MIN(I2,Inputs!B21*Decisions!I3)</f>
-        <v>172.973836798469</v>
+        <v>163.690528423469</v>
       </c>
       <c r="J3" s="10" t="n">
         <f aca="false">MIN(J2,Inputs!B21*Decisions!J3)</f>
-        <v>169.509589732972</v>
+        <v>156.098263019097</v>
       </c>
       <c r="K3" s="10" t="n">
         <f aca="false">MIN(K2,Inputs!B21*Decisions!K3)</f>
-        <v>165.652447220863</v>
+        <v>153.139679396817</v>
       </c>
       <c r="L3" s="10" t="n">
         <f aca="false">MIN(L2,Inputs!B21*Decisions!L3)</f>
-        <v>161.428733257065</v>
+        <v>150.75432087723</v>
       </c>
       <c r="M3" s="10" t="n">
         <f aca="false">MIN(M2,Inputs!B21*Decisions!M3)</f>
-        <v>156.238008128841</v>
+        <v>148.153781378456</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3093,27 +3093,27 @@
       </c>
       <c r="H4" s="11" t="n">
         <f aca="false">G4+G3</f>
-        <v>2536.81611398844</v>
+        <v>2536.44111398844</v>
       </c>
       <c r="I4" s="11" t="n">
         <f aca="false">H4+H3</f>
-        <v>2714.84273435121</v>
+        <v>2709.74285935121</v>
       </c>
       <c r="J4" s="11" t="n">
         <f aca="false">I4+I3</f>
-        <v>2887.81657114968</v>
+        <v>2873.43338777468</v>
       </c>
       <c r="K4" s="11" t="n">
         <f aca="false">J4+J3</f>
-        <v>3057.32616088265</v>
+        <v>3029.53165079378</v>
       </c>
       <c r="L4" s="11" t="n">
         <f aca="false">K4+K3</f>
-        <v>3222.97860810351</v>
+        <v>3182.67133019059</v>
       </c>
       <c r="M4" s="11" t="n">
         <f aca="false">L4+L3</f>
-        <v>3384.40734136058</v>
+        <v>3333.42565106782</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3142,27 +3142,27 @@
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">Inputs!B25*(H4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.57115583295252</v>
+        <v>1.57119067388082</v>
       </c>
       <c r="I5" s="12" t="n">
         <f aca="false">Inputs!B25*(I4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.55525250211784</v>
+        <v>1.55569121107628</v>
       </c>
       <c r="J5" s="12" t="n">
         <f aca="false">Inputs!B25*(J4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.54090963102866</v>
+        <v>1.54206414786714</v>
       </c>
       <c r="K5" s="12" t="n">
         <f aca="false">Inputs!B25*(K4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.52778184312453</v>
+        <v>1.52987619181317</v>
       </c>
       <c r="L5" s="12" t="n">
         <f aca="false">Inputs!B25*(L4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.51573750493053</v>
+        <v>1.51860155917332</v>
       </c>
       <c r="M5" s="12" t="n">
         <f aca="false">Inputs!B25*(M4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.50466637546077</v>
+        <v>1.5080960216442</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3191,27 +3191,27 @@
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6*(1-Inputs!B29)+G8/MAX(G3,1)</f>
-        <v>1.99603662659874</v>
+        <v>1.99614526365703</v>
       </c>
       <c r="I6" s="12" t="n">
         <f aca="false">H6*(1-Inputs!B29)+H8/MAX(H3,1)</f>
-        <v>2.04123505499145</v>
+        <v>2.04311908611372</v>
       </c>
       <c r="J6" s="12" t="n">
         <f aca="false">I6*(1-Inputs!B29)+I8/MAX(I3,1)</f>
-        <v>2.12257219630547</v>
+        <v>2.13020786094338</v>
       </c>
       <c r="K6" s="12" t="n">
         <f aca="false">J6*(1-Inputs!B29)+J8/MAX(J3,1)</f>
-        <v>2.23113264180738</v>
+        <v>2.24984264847517</v>
       </c>
       <c r="L6" s="12" t="n">
         <f aca="false">K6*(1-Inputs!B29)+K8/MAX(K3,1)</f>
-        <v>2.36601790642597</v>
+        <v>2.39738506380598</v>
       </c>
       <c r="M6" s="12" t="n">
         <f aca="false">L6*(1-Inputs!B29)+L8/MAX(L3,1)</f>
-        <v>2.52646373748986</v>
+        <v>2.57055315793648</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3331,31 +3331,31 @@
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">G6*G3</f>
-        <v>361.307637833258</v>
+        <v>360.57172563799</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">H6*H3</f>
-        <v>355.347654753688</v>
+        <v>345.935458189399</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">I6*I3</f>
-        <v>353.080259269405</v>
+        <v>334.43924283803</v>
       </c>
       <c r="J9" s="10" t="n">
         <f aca="false">J6*J3</f>
-        <v>359.796342174353</v>
+        <v>332.521746962887</v>
       </c>
       <c r="K9" s="10" t="n">
         <f aca="false">K6*K3</f>
-        <v>369.59258218974</v>
+        <v>344.540181880773</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">L6*L3</f>
-        <v>381.943273497876</v>
+        <v>361.416157175286</v>
       </c>
       <c r="M9" s="10" t="n">
         <f aca="false">M6*M3</f>
-        <v>394.729661955163</v>
+        <v>380.83717058262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3380,31 +3380,31 @@
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">G5*G3</f>
-        <v>292.556618313393</v>
+        <v>291.96073834663</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">H5*H3</f>
-        <v>279.707563003798</v>
+        <v>272.290086081261</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">I5*I3</f>
-        <v>269.017992481742</v>
+        <v>254.651916404823</v>
       </c>
       <c r="J10" s="10" t="n">
         <f aca="false">J5*J3</f>
-        <v>261.198959371253</v>
+        <v>240.713534946084</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">K5*K3</f>
-        <v>253.080801133179</v>
+        <v>234.284749531092</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">L5*L3</f>
-        <v>244.683585371159</v>
+        <v>228.935746736278</v>
       </c>
       <c r="M10" s="10" t="n">
         <f aca="false">M5*M3</f>
-        <v>235.086077400434</v>
+        <v>223.430128288394</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3429,31 +3429,31 @@
       </c>
       <c r="G11" s="10" t="n">
         <f aca="false">G9-G10-Inputs!F39-Decisions!G19</f>
-        <v>-1.24898048013472</v>
+        <v>-1.38901270864005</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">H9-H10-Inputs!G39-Decisions!H19</f>
-        <v>0.640091749889621</v>
+        <v>-1.3546278918617</v>
       </c>
       <c r="I11" s="10" t="n">
         <f aca="false">I9-I10-Inputs!H39-Decisions!I19</f>
-        <v>4.06226678766274</v>
+        <v>-0.212673566792859</v>
       </c>
       <c r="J11" s="10" t="n">
         <f aca="false">J9-J10-Inputs!I39-Decisions!J19</f>
-        <v>13.5973828031006</v>
+        <v>6.80821201680257</v>
       </c>
       <c r="K11" s="10" t="n">
         <f aca="false">K9-K10-Inputs!J39-Decisions!K19</f>
-        <v>26.5117810565617</v>
+        <v>20.2554323496811</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">L9-L10-Inputs!K39-Decisions!L19</f>
-        <v>42.2596881267166</v>
+        <v>37.4804104390084</v>
       </c>
       <c r="M11" s="10" t="n">
         <f aca="false">M9-M10-Inputs!L39-Decisions!M19</f>
-        <v>59.64358455473</v>
+        <v>57.4070422942264</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,39 +3473,39 @@
       </c>
       <c r="E13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*D13+(Decisions!D12)/Inputs!C22</f>
-        <v>135.38668</v>
+        <v>133.38668</v>
       </c>
       <c r="F13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*E13+(Decisions!E12)/Inputs!C22</f>
-        <v>161.31577244</v>
+        <v>134.44977244</v>
       </c>
       <c r="G13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*F13+(Decisions!F12)/Inputs!C22</f>
-        <v>190.50761568652</v>
+        <v>136.44163768652</v>
       </c>
       <c r="H13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*G13+(Decisions!G12)/Inputs!C22</f>
-        <v>222.743605435523</v>
+        <v>145.300047961523</v>
       </c>
       <c r="I13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*H13+(Decisions!H12)/Inputs!C22</f>
-        <v>247.819783871343</v>
+        <v>175.564944748101</v>
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*I13+(Decisions!I12)/Inputs!C22</f>
-        <v>271.215858351963</v>
+        <v>206.802093449978</v>
       </c>
       <c r="K13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*J13+(Decisions!J12)/Inputs!C22</f>
-        <v>283.044395842382</v>
+        <v>232.94635318883</v>
       </c>
       <c r="L13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*K13+(Decisions!K12)/Inputs!C22</f>
-        <v>289.080421320942</v>
+        <v>250.338947525178</v>
       </c>
       <c r="M13" s="10" t="n">
         <f aca="false">(1-Inputs!C24)*L13+(Decisions!L12)/Inputs!C22</f>
-        <v>289.712033092439</v>
+        <v>259.566238040991</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3522,39 +3522,39 @@
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">MIN(E13,Inputs!C21*Decisions!E4)</f>
-        <v>135.38668</v>
+        <v>133.38668</v>
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">MIN(F13,Inputs!C21*Decisions!F4)</f>
-        <v>161.31577244</v>
+        <v>134.44977244</v>
       </c>
       <c r="G14" s="10" t="n">
         <f aca="false">MIN(G13,Inputs!C21*Decisions!G4)</f>
-        <v>190.50761568652</v>
+        <v>136.44163768652</v>
       </c>
       <c r="H14" s="10" t="n">
         <f aca="false">MIN(H13,Inputs!C21*Decisions!H4)</f>
-        <v>222.743605435523</v>
+        <v>145.300047961523</v>
       </c>
       <c r="I14" s="10" t="n">
         <f aca="false">MIN(I13,Inputs!C21*Decisions!I4)</f>
-        <v>247.819783871343</v>
+        <v>175.564944748101</v>
       </c>
       <c r="J14" s="10" t="n">
         <f aca="false">MIN(J13,Inputs!C21*Decisions!J4)</f>
-        <v>271.215858351963</v>
+        <v>206.802093449978</v>
       </c>
       <c r="K14" s="10" t="n">
         <f aca="false">MIN(K13,Inputs!C21*Decisions!K4)</f>
-        <v>283.044395842382</v>
+        <v>232.94635318883</v>
       </c>
       <c r="L14" s="10" t="n">
         <f aca="false">MIN(L13,Inputs!C21*Decisions!L4)</f>
-        <v>289.080421320942</v>
+        <v>250.338947525178</v>
       </c>
       <c r="M14" s="10" t="n">
         <f aca="false">MIN(M13,Inputs!C21*Decisions!M4)</f>
-        <v>289.712033092439</v>
+        <v>259.566238040991</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,35 +3575,35 @@
       </c>
       <c r="F15" s="11" t="n">
         <f aca="false">E15+E14</f>
-        <v>1183.19668</v>
+        <v>1181.19668</v>
       </c>
       <c r="G15" s="11" t="n">
         <f aca="false">F15+F14</f>
-        <v>1344.51245244</v>
+        <v>1315.64645244</v>
       </c>
       <c r="H15" s="11" t="n">
         <f aca="false">G15+G14</f>
-        <v>1535.02006812652</v>
+        <v>1452.08809012652</v>
       </c>
       <c r="I15" s="11" t="n">
         <f aca="false">H15+H14</f>
-        <v>1757.76367356204</v>
+        <v>1597.38813808804</v>
       </c>
       <c r="J15" s="11" t="n">
         <f aca="false">I15+I14</f>
-        <v>2005.58345743339</v>
+        <v>1772.95308283614</v>
       </c>
       <c r="K15" s="11" t="n">
         <f aca="false">J15+J14</f>
-        <v>2276.79931578535</v>
+        <v>1979.75517628612</v>
       </c>
       <c r="L15" s="11" t="n">
         <f aca="false">K15+K14</f>
-        <v>2559.84371162773</v>
+        <v>2212.70152947495</v>
       </c>
       <c r="M15" s="11" t="n">
         <f aca="false">L15+L14</f>
-        <v>2848.92413294867</v>
+        <v>2463.04047700013</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,35 +3624,35 @@
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">Inputs!C25*(F15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>1.04953433410695</v>
+        <v>1.04974742375136</v>
       </c>
       <c r="G16" s="12" t="n">
         <f aca="false">Inputs!C25*(G15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>1.03356002586595</v>
+        <v>1.03625533560432</v>
       </c>
       <c r="H16" s="12" t="n">
         <f aca="false">Inputs!C25*(H15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>1.01725491453862</v>
+        <v>1.024057465529</v>
       </c>
       <c r="I16" s="12" t="n">
         <f aca="false">Inputs!C25*(I15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>1.00084822986055</v>
+        <v>1.01240487790922</v>
       </c>
       <c r="J16" s="12" t="n">
         <f aca="false">Inputs!C25*(J15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>0.985132382158583</v>
+        <v>0.999815382923979</v>
       </c>
       <c r="K16" s="12" t="n">
         <f aca="false">Inputs!C25*(K15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>0.970251925598136</v>
+        <v>0.986665868781465</v>
       </c>
       <c r="L16" s="12" t="n">
         <f aca="false">Inputs!C25*(L15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>0.956704616248162</v>
+        <v>0.973582464933597</v>
       </c>
       <c r="M16" s="12" t="n">
         <f aca="false">Inputs!C25*(M15/Inputs!C27)^(-Inputs!C26)</f>
-        <v>0.944499598201517</v>
+        <v>0.961140544316875</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3673,35 +3673,35 @@
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">E17*(1-Inputs!C29)+E19/MAX(E14,1)</f>
-        <v>1.48890431997027</v>
+        <v>1.4897349408759</v>
       </c>
       <c r="G17" s="12" t="n">
         <f aca="false">F17*(1-Inputs!C29)+F19/MAX(F14,1)</f>
-        <v>1.58745168147476</v>
+        <v>1.61242449135774</v>
       </c>
       <c r="H17" s="12" t="n">
         <f aca="false">G17*(1-Inputs!C29)+G19/MAX(G14,1)</f>
-        <v>1.72898762679644</v>
+        <v>1.81910606528527</v>
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">H17*(1-Inputs!C29)+H19/MAX(H14,1)</f>
-        <v>1.88992686392388</v>
+        <v>2.07829563576619</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">I17*(1-Inputs!C29)+I19/MAX(I14,1)</f>
-        <v>2.05829349044555</v>
+        <v>2.32479622382573</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">J17*(1-Inputs!C29)+J19/MAX(J14,1)</f>
-        <v>2.22237450227922</v>
+        <v>2.54560351039253</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">K17*(1-Inputs!C29)+K19/MAX(K14,1)</f>
-        <v>2.38147777701807</v>
+        <v>2.7412447537946</v>
       </c>
       <c r="M17" s="12" t="n">
         <f aca="false">L17*(1-Inputs!C29)+L19/MAX(L14,1)</f>
-        <v>2.53352775263367</v>
+        <v>2.91695710513365</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3814,39 +3814,39 @@
       </c>
       <c r="E20" s="10" t="n">
         <f aca="false">E17*E14</f>
-        <v>197.0333124045</v>
+        <v>194.1226374045</v>
       </c>
       <c r="F20" s="10" t="n">
         <f aca="false">F17*F14</f>
-        <v>240.183750465257</v>
+        <v>200.294523796682</v>
       </c>
       <c r="G20" s="10" t="n">
         <f aca="false">G17*G14</f>
-        <v>302.421634855314</v>
+        <v>220.001838246704</v>
       </c>
       <c r="H20" s="10" t="n">
         <f aca="false">H17*H14</f>
-        <v>385.120937746048</v>
+        <v>264.316198533048</v>
       </c>
       <c r="I20" s="10" t="n">
         <f aca="false">I17*I14</f>
-        <v>468.361266950262</v>
+        <v>364.875858463511</v>
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">J17*J14</f>
-        <v>558.241835751447</v>
+        <v>480.772725931765</v>
       </c>
       <c r="K20" s="10" t="n">
         <f aca="false">K17*K14</f>
-        <v>629.030648333135</v>
+        <v>592.989054410623</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">L17*L14</f>
-        <v>688.438599146845</v>
+        <v>686.240326573857</v>
       </c>
       <c r="M20" s="10" t="n">
         <f aca="false">M17*M14</f>
-        <v>733.99347611162</v>
+        <v>757.143582306482</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3863,39 +3863,39 @@
       </c>
       <c r="E21" s="10" t="n">
         <f aca="false">E16*E14</f>
-        <v>144.180164727801</v>
+        <v>142.050262957142</v>
       </c>
       <c r="F21" s="10" t="n">
         <f aca="false">F16*F14</f>
-        <v>169.306441808764</v>
+        <v>141.138302242846</v>
       </c>
       <c r="G21" s="10" t="n">
         <f aca="false">G16*G14</f>
-        <v>196.901056196621</v>
+        <v>141.388375051248</v>
       </c>
       <c r="H21" s="10" t="n">
         <f aca="false">H16*H14</f>
-        <v>226.587027311338</v>
+        <v>148.79559885672</v>
       </c>
       <c r="I21" s="10" t="n">
         <f aca="false">I16*I14</f>
-        <v>248.029992012057</v>
+        <v>177.74280645284</v>
       </c>
       <c r="J21" s="10" t="n">
         <f aca="false">J16*J14</f>
-        <v>267.183524617454</v>
+        <v>206.763914252171</v>
       </c>
       <c r="K21" s="10" t="n">
         <f aca="false">K16*K14</f>
-        <v>274.624370095832</v>
+        <v>229.840215948531</v>
       </c>
       <c r="L21" s="10" t="n">
         <f aca="false">L16*L14</f>
-        <v>276.564573544709</v>
+        <v>243.725609600445</v>
       </c>
       <c r="M21" s="10" t="n">
         <f aca="false">M16*M14</f>
-        <v>273.632898849953</v>
+        <v>249.479635317002</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,39 +3912,39 @@
       </c>
       <c r="E22" s="10" t="n">
         <f aca="false">E20-E21-Inputs!D40-Decisions!E20</f>
-        <v>15.8531476766989</v>
+        <v>15.0723744473576</v>
       </c>
       <c r="F22" s="10" t="n">
         <f aca="false">F20-F21-Inputs!E40-Decisions!F20</f>
-        <v>30.8773086564933</v>
+        <v>19.1562215538352</v>
       </c>
       <c r="G22" s="10" t="n">
         <f aca="false">G20-G21-Inputs!F40-Decisions!G20</f>
-        <v>61.5205786586931</v>
+        <v>34.6134631954567</v>
       </c>
       <c r="H22" s="10" t="n">
         <f aca="false">H20-H21-Inputs!G40-Decisions!H20</f>
-        <v>110.53391043471</v>
+        <v>67.5205996763273</v>
       </c>
       <c r="I22" s="10" t="n">
         <f aca="false">I20-I21-Inputs!H40-Decisions!I20</f>
-        <v>168.331274938205</v>
+        <v>135.133052010671</v>
       </c>
       <c r="J22" s="10" t="n">
         <f aca="false">J20-J21-Inputs!I40-Decisions!J20</f>
-        <v>235.058311133993</v>
+        <v>218.008811679595</v>
       </c>
       <c r="K22" s="10" t="n">
         <f aca="false">K20-K21-Inputs!J40-Decisions!K20</f>
-        <v>294.406278237303</v>
+        <v>303.148838462092</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">L20-L21-Inputs!K40-Decisions!L20</f>
-        <v>347.874025602136</v>
+        <v>378.514716973411</v>
       </c>
       <c r="M22" s="10" t="n">
         <f aca="false">M20-M21-Inputs!L40-Decisions!M20</f>
-        <v>392.360577261666</v>
+        <v>439.66394698948</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3968,35 +3968,35 @@
       </c>
       <c r="F24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*E24+(Decisions!D13)/Inputs!D22</f>
-        <v>37.12584948</v>
+        <v>36.92584948</v>
       </c>
       <c r="G24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*F24+(Decisions!E13)/Inputs!D22</f>
-        <v>39.63841756484</v>
+        <v>36.05181756484</v>
       </c>
       <c r="H24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*G24+(Decisions!F13)/Inputs!D22</f>
-        <v>42.9826435879957</v>
+        <v>35.2363457879957</v>
       </c>
       <c r="I24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*H24+(Decisions!G13)/Inputs!D22</f>
-        <v>47.1028064676</v>
+        <v>35.6755106202</v>
       </c>
       <c r="J24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*I24+(Decisions!H13)/Inputs!D22</f>
-        <v>50.9469184342708</v>
+        <v>39.8852514086466</v>
       </c>
       <c r="K24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*J24+(Decisions!I13)/Inputs!D22</f>
-        <v>53.5334748991747</v>
+        <v>44.2129395642673</v>
       </c>
       <c r="L24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*K24+(Decisions!J13)/Inputs!D22</f>
-        <v>54.94673208093</v>
+        <v>48.0506726134614</v>
       </c>
       <c r="M24" s="10" t="n">
         <f aca="false">(1-Inputs!D24)*L24+(Decisions!K13)/Inputs!D22</f>
-        <v>55.2653010315077</v>
+        <v>50.4312775483595</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,35 +4017,35 @@
       </c>
       <c r="F25" s="10" t="n">
         <f aca="false">MIN(F24,Inputs!D21*Decisions!F5)</f>
-        <v>37.12584948</v>
+        <v>36.92584948</v>
       </c>
       <c r="G25" s="10" t="n">
         <f aca="false">MIN(G24,Inputs!D21*Decisions!G5)</f>
-        <v>39.63841756484</v>
+        <v>36.05181756484</v>
       </c>
       <c r="H25" s="10" t="n">
         <f aca="false">MIN(H24,Inputs!D21*Decisions!H5)</f>
-        <v>42.9826435879957</v>
+        <v>35.2363457879957</v>
       </c>
       <c r="I25" s="10" t="n">
         <f aca="false">MIN(I24,Inputs!D21*Decisions!I5)</f>
-        <v>47.1028064676</v>
+        <v>35.6755106202</v>
       </c>
       <c r="J25" s="10" t="n">
         <f aca="false">MIN(J24,Inputs!D21*Decisions!J5)</f>
-        <v>50.9469184342708</v>
+        <v>39.8852514086466</v>
       </c>
       <c r="K25" s="10" t="n">
         <f aca="false">MIN(K24,Inputs!D21*Decisions!K5)</f>
-        <v>53.5334748991747</v>
+        <v>44.2129395642673</v>
       </c>
       <c r="L25" s="10" t="n">
         <f aca="false">MIN(L24,Inputs!D21*Decisions!L5)</f>
-        <v>54.94673208093</v>
+        <v>48.0506726134614</v>
       </c>
       <c r="M25" s="10" t="n">
         <f aca="false">MIN(M24,Inputs!D21*Decisions!M5)</f>
-        <v>55.2653010315077</v>
+        <v>50.4312775483595</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4070,31 +4070,31 @@
       </c>
       <c r="G26" s="11" t="n">
         <f aca="false">F26+F25</f>
-        <v>351.41540948</v>
+        <v>351.21540948</v>
       </c>
       <c r="H26" s="11" t="n">
         <f aca="false">G26+G25</f>
-        <v>391.05382704484</v>
+        <v>387.26722704484</v>
       </c>
       <c r="I26" s="11" t="n">
         <f aca="false">H26+H25</f>
-        <v>434.036470632836</v>
+        <v>422.503572832836</v>
       </c>
       <c r="J26" s="11" t="n">
         <f aca="false">I26+I25</f>
-        <v>481.139277100436</v>
+        <v>458.179083453036</v>
       </c>
       <c r="K26" s="11" t="n">
         <f aca="false">J26+J25</f>
-        <v>532.086195534707</v>
+        <v>498.064334861682</v>
       </c>
       <c r="L26" s="11" t="n">
         <f aca="false">K26+K25</f>
-        <v>585.619670433881</v>
+        <v>542.27727442595</v>
       </c>
       <c r="M26" s="11" t="n">
         <f aca="false">L26+L25</f>
-        <v>640.566402514811</v>
+        <v>590.327947039411</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4119,31 +4119,31 @@
       </c>
       <c r="G27" s="12" t="n">
         <f aca="false">Inputs!D25*(G26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.49535768148367</v>
+        <v>1.49545983985829</v>
       </c>
       <c r="H27" s="12" t="n">
         <f aca="false">Inputs!D25*(H26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.47630196318975</v>
+        <v>1.47802674470777</v>
       </c>
       <c r="I27" s="12" t="n">
         <f aca="false">Inputs!D25*(I26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.45794263164366</v>
+        <v>1.46266185611919</v>
       </c>
       <c r="J27" s="12" t="n">
         <f aca="false">Inputs!D25*(J26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.44002849122153</v>
+        <v>1.44850284000839</v>
       </c>
       <c r="K27" s="12" t="n">
         <f aca="false">Inputs!D25*(K26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.42274065965199</v>
+        <v>1.43406662581304</v>
       </c>
       <c r="L27" s="12" t="n">
         <f aca="false">Inputs!D25*(L26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.40646750742239</v>
+        <v>1.41950528431624</v>
       </c>
       <c r="M27" s="12" t="n">
         <f aca="false">Inputs!D25*(M26/Inputs!D27)^(-Inputs!D26)</f>
-        <v>1.39141244481563</v>
+        <v>1.40511665279785</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4168,31 +4168,31 @@
       </c>
       <c r="G28" s="12" t="n">
         <f aca="false">F28*(1-Inputs!D29)+F30/MAX(F25,1)</f>
-        <v>1.9255425518309</v>
+        <v>1.92598021938882</v>
       </c>
       <c r="H28" s="12" t="n">
         <f aca="false">G28*(1-Inputs!D29)+G30/MAX(G25,1)</f>
-        <v>1.98794390278764</v>
+        <v>1.99841202522623</v>
       </c>
       <c r="I28" s="12" t="n">
         <f aca="false">H28*(1-Inputs!D29)+H30/MAX(H25,1)</f>
-        <v>2.06451104804322</v>
+        <v>2.10034272140723</v>
       </c>
       <c r="J28" s="12" t="n">
         <f aca="false">I28*(1-Inputs!D29)+I30/MAX(I25,1)</f>
-        <v>2.21429224458251</v>
+        <v>2.31060976141086</v>
       </c>
       <c r="K28" s="12" t="n">
         <f aca="false">J28*(1-Inputs!D29)+J30/MAX(J25,1)</f>
-        <v>2.41339697916228</v>
+        <v>2.57528942625781</v>
       </c>
       <c r="L28" s="12" t="n">
         <f aca="false">K28*(1-Inputs!D29)+K30/MAX(K25,1)</f>
-        <v>2.65653549188539</v>
+        <v>2.87662152079908</v>
       </c>
       <c r="M28" s="12" t="n">
         <f aca="false">L28*(1-Inputs!D29)+L30/MAX(L25,1)</f>
-        <v>2.94191444942161</v>
+        <v>3.20618044599483</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4308,35 +4308,35 @@
       </c>
       <c r="F31" s="10" t="n">
         <f aca="false">F28*F25</f>
-        <v>69.8851050475603</v>
+        <v>69.5086282475603</v>
       </c>
       <c r="G31" s="10" t="n">
         <f aca="false">G28*G25</f>
-        <v>76.3254597083408</v>
+        <v>69.4350875028964</v>
       </c>
       <c r="H31" s="10" t="n">
         <f aca="false">H28*H25</f>
-        <v>85.4470842464502</v>
+        <v>70.4167371477603</v>
       </c>
       <c r="I31" s="10" t="n">
         <f aca="false">I28*I25</f>
-        <v>97.2442643462017</v>
+        <v>74.9307990636234</v>
       </c>
       <c r="J31" s="10" t="n">
         <f aca="false">J28*J25</f>
-        <v>112.811366374384</v>
+        <v>92.1592512411451</v>
       </c>
       <c r="K31" s="10" t="n">
         <f aca="false">K28*K25</f>
-        <v>129.197526605728</v>
+        <v>113.861115763633</v>
       </c>
       <c r="L31" s="10" t="n">
         <f aca="false">L28*L25</f>
-        <v>145.967943936108</v>
+        <v>138.223598928754</v>
       </c>
       <c r="M31" s="10" t="n">
         <f aca="false">M28*M25</f>
-        <v>162.585787656227</v>
+        <v>161.691775942088</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4357,35 +4357,35 @@
       </c>
       <c r="F32" s="10" t="n">
         <f aca="false">F27*F25</f>
-        <v>56.2652673897627</v>
+        <v>55.9621617737144</v>
       </c>
       <c r="G32" s="10" t="n">
         <f aca="false">G27*G25</f>
-        <v>59.2736121874406</v>
+        <v>53.9140453221158</v>
       </c>
       <c r="H32" s="10" t="n">
         <f aca="false">H27*H25</f>
-        <v>63.4553611120435</v>
+        <v>52.0802614604287</v>
       </c>
       <c r="I32" s="10" t="n">
         <f aca="false">I27*I25</f>
-        <v>68.6731896191747</v>
+        <v>52.1812085817415</v>
       </c>
       <c r="J32" s="10" t="n">
         <f aca="false">J27*J25</f>
-        <v>73.3650140852892</v>
+        <v>57.7738999398731</v>
       </c>
       <c r="K32" s="10" t="n">
         <f aca="false">K27*K25</f>
-        <v>76.164251391515</v>
+        <v>63.4043010582046</v>
       </c>
       <c r="L32" s="10" t="n">
         <f aca="false">L27*L25</f>
-        <v>77.2807933108713</v>
+        <v>68.208183689758</v>
       </c>
       <c r="M32" s="10" t="n">
         <f aca="false">M27*M25</f>
-        <v>76.8968276217221</v>
+        <v>70.8618279050701</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4406,35 +4406,35 @@
       </c>
       <c r="F33" s="10" t="n">
         <f aca="false">F31-F32-Inputs!E41-Decisions!F21</f>
-        <v>-11.3801623422023</v>
+        <v>-11.453533526154</v>
       </c>
       <c r="G33" s="10" t="n">
         <f aca="false">G31-G32-Inputs!F41-Decisions!G21</f>
-        <v>-10.9481524790998</v>
+        <v>-12.4789578192194</v>
       </c>
       <c r="H33" s="10" t="n">
         <f aca="false">H31-H32-Inputs!G41-Decisions!H21</f>
-        <v>-9.0082768655934</v>
+        <v>-12.6635243126684</v>
       </c>
       <c r="I33" s="10" t="n">
         <f aca="false">I31-I32-Inputs!H41-Decisions!I21</f>
-        <v>-5.42892527297296</v>
+        <v>-11.2504095181181</v>
       </c>
       <c r="J33" s="10" t="n">
         <f aca="false">J31-J32-Inputs!I41-Decisions!J21</f>
-        <v>2.44635228909446</v>
+        <v>-2.61464869872807</v>
       </c>
       <c r="K33" s="10" t="n">
         <f aca="false">K31-K32-Inputs!J41-Decisions!K21</f>
-        <v>13.0332752142127</v>
+        <v>10.4568147054286</v>
       </c>
       <c r="L33" s="10" t="n">
         <f aca="false">L31-L32-Inputs!K41-Decisions!L21</f>
-        <v>25.6871506252367</v>
+        <v>27.0154152389962</v>
       </c>
       <c r="M33" s="10" t="n">
         <f aca="false">M31-M32-Inputs!L41-Decisions!M21</f>
-        <v>39.6889600345054</v>
+        <v>44.8299480370181</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4462,31 +4462,31 @@
       </c>
       <c r="G35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*F35+(Decisions!D14)/Inputs!E22</f>
-        <v>6.60837326139267</v>
+        <v>6.47503992805934</v>
       </c>
       <c r="H35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*G35+(Decisions!E14)/Inputs!E22</f>
-        <v>8.16561225287936</v>
+        <v>6.70787891954603</v>
       </c>
       <c r="I35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*H35+(Decisions!F14)/Inputs!E22</f>
-        <v>9.95184956526978</v>
+        <v>6.99178436526978</v>
       </c>
       <c r="J35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*I35+(Decisions!G14)/Inputs!E22</f>
-        <v>11.9517423110634</v>
+        <v>7.7233348127967</v>
       </c>
       <c r="K35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*J35+(Decisions!H14)/Inputs!E22</f>
-        <v>13.4843089095555</v>
+        <v>9.60587138033933</v>
       </c>
       <c r="L35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*K35+(Decisions!I14)/Inputs!E22</f>
-        <v>14.5808602126152</v>
+        <v>11.5622779978566</v>
       </c>
       <c r="M35" s="10" t="n">
         <f aca="false">(1-Inputs!E24)*L35+(Decisions!J14)/Inputs!E22</f>
-        <v>15.2706092450367</v>
+        <v>13.2542720386669</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4511,31 +4511,31 @@
       </c>
       <c r="G36" s="10" t="n">
         <f aca="false">MIN(G35,Inputs!E21*Decisions!G6)</f>
-        <v>6.60837326139267</v>
+        <v>6.47503992805934</v>
       </c>
       <c r="H36" s="10" t="n">
         <f aca="false">MIN(H35,Inputs!E21*Decisions!H6)</f>
-        <v>8.16561225287936</v>
+        <v>6.70787891954603</v>
       </c>
       <c r="I36" s="10" t="n">
         <f aca="false">MIN(I35,Inputs!E21*Decisions!I6)</f>
-        <v>9.95184956526978</v>
+        <v>6.99178436526978</v>
       </c>
       <c r="J36" s="10" t="n">
         <f aca="false">MIN(J35,Inputs!E21*Decisions!J6)</f>
-        <v>11.9517423110634</v>
+        <v>7.7233348127967</v>
       </c>
       <c r="K36" s="10" t="n">
         <f aca="false">MIN(K35,Inputs!E21*Decisions!K6)</f>
-        <v>13.4843089095555</v>
+        <v>9.60587138033933</v>
       </c>
       <c r="L36" s="10" t="n">
         <f aca="false">MIN(L35,Inputs!E21*Decisions!L6)</f>
-        <v>14.5808602126152</v>
+        <v>11.5622779978566</v>
       </c>
       <c r="M36" s="10" t="n">
         <f aca="false">MIN(M35,Inputs!E21*Decisions!M6)</f>
-        <v>15.2706092450367</v>
+        <v>13.2542720386669</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4564,27 +4564,27 @@
       </c>
       <c r="H37" s="11" t="n">
         <f aca="false">G37+G36</f>
-        <v>54.3689713500593</v>
+        <v>54.235638016726</v>
       </c>
       <c r="I37" s="11" t="n">
         <f aca="false">H37+H36</f>
-        <v>62.5345836029387</v>
+        <v>60.943516936272</v>
       </c>
       <c r="J37" s="11" t="n">
         <f aca="false">I37+I36</f>
-        <v>72.4864331682085</v>
+        <v>67.9353013015418</v>
       </c>
       <c r="K37" s="11" t="n">
         <f aca="false">J37+J36</f>
-        <v>84.4381754792719</v>
+        <v>75.6586361143385</v>
       </c>
       <c r="L37" s="11" t="n">
         <f aca="false">K37+K36</f>
-        <v>97.9224843888273</v>
+        <v>85.2645074946778</v>
       </c>
       <c r="M37" s="11" t="n">
         <f aca="false">L37+L36</f>
-        <v>112.503344601443</v>
+        <v>96.8267854925344</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4613,27 +4613,27 @@
       </c>
       <c r="H38" s="12" t="n">
         <f aca="false">Inputs!E25*(H37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>4.10921642951723</v>
+        <v>4.11123487184404</v>
       </c>
       <c r="I38" s="12" t="n">
         <f aca="false">Inputs!E25*(I37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>3.99581328658799</v>
+        <v>4.01646268522398</v>
       </c>
       <c r="J38" s="12" t="n">
         <f aca="false">Inputs!E25*(J37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>3.87951908877181</v>
+        <v>3.93015915582004</v>
       </c>
       <c r="K38" s="12" t="n">
         <f aca="false">Inputs!E25*(K37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>3.76288955075088</v>
+        <v>3.84642738055001</v>
       </c>
       <c r="L38" s="12" t="n">
         <f aca="false">Inputs!E25*(L37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>3.65302592566066</v>
+        <v>3.75556758168816</v>
       </c>
       <c r="M38" s="12" t="n">
         <f aca="false">Inputs!E25*(M37/Inputs!E27)^(-Inputs!E26)</f>
-        <v>3.55300773009273</v>
+        <v>3.66125633616422</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4662,27 +4662,27 @@
       </c>
       <c r="H39" s="12" t="n">
         <f aca="false">G39*(1-Inputs!E29)+G41/MAX(G36,1)</f>
-        <v>6.98641630456163</v>
+        <v>7.0097865344174</v>
       </c>
       <c r="I39" s="12" t="n">
         <f aca="false">H39*(1-Inputs!E29)+H41/MAX(H36,1)</f>
-        <v>8.38432228069633</v>
+        <v>8.71895513165741</v>
       </c>
       <c r="J39" s="12" t="n">
         <f aca="false">I39*(1-Inputs!E29)+I41/MAX(I36,1)</f>
-        <v>9.94009363035691</v>
+        <v>10.9494579495948</v>
       </c>
       <c r="K39" s="12" t="n">
         <f aca="false">J39*(1-Inputs!E29)+J41/MAX(J36,1)</f>
-        <v>12.011422828025</v>
+        <v>14.1769715762062</v>
       </c>
       <c r="L39" s="12" t="n">
         <f aca="false">K39*(1-Inputs!E29)+K41/MAX(K36,1)</f>
-        <v>14.5321431369933</v>
+        <v>17.7288710157733</v>
       </c>
       <c r="M39" s="12" t="n">
         <f aca="false">L39*(1-Inputs!E29)+L41/MAX(L36,1)</f>
-        <v>17.4171268518261</v>
+        <v>21.3700280033014</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4801,31 +4801,31 @@
       </c>
       <c r="G42" s="10" t="n">
         <f aca="false">G39*G36</f>
-        <v>38.8631625125858</v>
+        <v>38.0790429120858</v>
       </c>
       <c r="H42" s="10" t="n">
         <f aca="false">H39*H36</f>
-        <v>57.0483665802446</v>
+        <v>47.0207993247361</v>
       </c>
       <c r="I42" s="10" t="n">
         <f aca="false">I39*I36</f>
-        <v>83.4395140442294</v>
+        <v>60.961054171011</v>
       </c>
       <c r="J42" s="10" t="n">
         <f aca="false">J39*J36</f>
-        <v>118.801437617868</v>
+        <v>84.5663297633593</v>
       </c>
       <c r="K42" s="10" t="n">
         <f aca="false">K39*K36</f>
-        <v>161.965735856375</v>
+        <v>136.182165523763</v>
       </c>
       <c r="L42" s="10" t="n">
         <f aca="false">L39*L36</f>
-        <v>211.891147670215</v>
+        <v>204.986135272513</v>
       </c>
       <c r="M42" s="10" t="n">
         <f aca="false">M39*M36</f>
-        <v>265.970138325472</v>
+        <v>283.244164629685</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4850,31 +4850,31 @@
       </c>
       <c r="G43" s="10" t="n">
         <f aca="false">G38*G36</f>
-        <v>27.8682599614727</v>
+        <v>27.3059781641397</v>
       </c>
       <c r="H43" s="10" t="n">
         <f aca="false">H38*H36</f>
-        <v>33.5542680265991</v>
+        <v>27.5776657301451</v>
       </c>
       <c r="I43" s="10" t="n">
         <f aca="false">I38*I36</f>
-        <v>39.7657327190299</v>
+        <v>28.0822410062385</v>
       </c>
       <c r="J43" s="10" t="n">
         <f aca="false">J38*J36</f>
-        <v>46.367012439852</v>
+        <v>30.3539350279766</v>
       </c>
       <c r="K43" s="10" t="n">
         <f aca="false">K38*K36</f>
-        <v>50.7399650948633</v>
+        <v>36.9482866913789</v>
       </c>
       <c r="L43" s="10" t="n">
         <f aca="false">L38*L36</f>
-        <v>53.2642603751175</v>
+        <v>43.4229164192165</v>
       </c>
       <c r="M43" s="10" t="n">
         <f aca="false">M38*M36</f>
-        <v>54.2565926908409</v>
+        <v>48.5272874828133</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4899,31 +4899,31 @@
       </c>
       <c r="G44" s="10" t="n">
         <f aca="false">G42-G43-Inputs!F42-Decisions!G22</f>
-        <v>-26.005097448887</v>
+        <v>-26.226935252054</v>
       </c>
       <c r="H44" s="10" t="n">
         <f aca="false">H42-H43-Inputs!G42-Decisions!H22</f>
-        <v>-19.5059014463545</v>
+        <v>-23.556866405409</v>
       </c>
       <c r="I44" s="10" t="n">
         <f aca="false">I42-I43-Inputs!H42-Decisions!I22</f>
-        <v>-6.32621867480042</v>
+        <v>-17.1211868352275</v>
       </c>
       <c r="J44" s="10" t="n">
         <f aca="false">J42-J43-Inputs!I42-Decisions!J22</f>
-        <v>14.4344251780161</v>
+        <v>-3.78760526461738</v>
       </c>
       <c r="K44" s="10" t="n">
         <f aca="false">K42-K43-Inputs!J42-Decisions!K22</f>
-        <v>45.225770761512</v>
+        <v>33.2338788323841</v>
       </c>
       <c r="L44" s="10" t="n">
         <f aca="false">L42-L43-Inputs!K42-Decisions!L22</f>
-        <v>84.6268872950972</v>
+        <v>87.5632188532965</v>
       </c>
       <c r="M44" s="10" t="n">
         <f aca="false">M42-M43-Inputs!L42-Decisions!M22</f>
-        <v>128.713545634631</v>
+        <v>151.716877146872</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4947,35 +4947,35 @@
       </c>
       <c r="F46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*E46+(Decisions!D15)/Inputs!F22</f>
-        <v>396.37218295</v>
+        <v>390.37218295</v>
       </c>
       <c r="G46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*F46+(Decisions!E15)/Inputs!F22</f>
-        <v>479.81524669235</v>
+        <v>400.21724669235</v>
       </c>
       <c r="H46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*G46+(Decisions!F15)/Inputs!F22</f>
-        <v>577.667625163963</v>
+        <v>411.402691163963</v>
       </c>
       <c r="I46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*H46+(Decisions!G15)/Inputs!F22</f>
-        <v>688.963894277977</v>
+        <v>447.838710855977</v>
       </c>
       <c r="J46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*I46+(Decisions!H15)/Inputs!F22</f>
-        <v>782.803313361353</v>
+        <v>557.833517228627</v>
       </c>
       <c r="K46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*J46+(Decisions!I15)/Inputs!F22</f>
-        <v>850.355491366142</v>
+        <v>670.458671574309</v>
       </c>
       <c r="L46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*K46+(Decisions!J15)/Inputs!F22</f>
-        <v>903.381673444611</v>
+        <v>769.53794057883</v>
       </c>
       <c r="M46" s="10" t="n">
         <f aca="false">(1-Inputs!F24)*L46+(Decisions!K15)/Inputs!F22</f>
-        <v>932.855101323822</v>
+        <v>835.978898560049</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4996,35 +4996,35 @@
       </c>
       <c r="F47" s="10" t="n">
         <f aca="false">MIN(F46,Inputs!F21*Decisions!F7)</f>
-        <v>396.37218295</v>
+        <v>390.37218295</v>
       </c>
       <c r="G47" s="10" t="n">
         <f aca="false">MIN(G46,Inputs!F21*Decisions!G7)</f>
-        <v>479.81524669235</v>
+        <v>400.21724669235</v>
       </c>
       <c r="H47" s="10" t="n">
         <f aca="false">MIN(H46,Inputs!F21*Decisions!H7)</f>
-        <v>577.667625163963</v>
+        <v>411.402691163963</v>
       </c>
       <c r="I47" s="10" t="n">
         <f aca="false">MIN(I46,Inputs!F21*Decisions!I7)</f>
-        <v>648</v>
+        <v>447.838710855977</v>
       </c>
       <c r="J47" s="10" t="n">
         <f aca="false">MIN(J46,Inputs!F21*Decisions!J7)</f>
-        <v>702</v>
+        <v>557.833517228627</v>
       </c>
       <c r="K47" s="10" t="n">
         <f aca="false">MIN(K46,Inputs!F21*Decisions!K7)</f>
-        <v>756</v>
+        <v>670.458671574309</v>
       </c>
       <c r="L47" s="10" t="n">
         <f aca="false">MIN(L46,Inputs!F21*Decisions!L7)</f>
-        <v>814.5</v>
+        <v>769.53794057883</v>
       </c>
       <c r="M47" s="10" t="n">
         <f aca="false">MIN(M46,Inputs!F21*Decisions!M7)</f>
-        <v>873</v>
+        <v>835.978898560049</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5049,31 +5049,31 @@
       </c>
       <c r="G48" s="11" t="n">
         <f aca="false">F48+F47</f>
-        <v>4435.59333295</v>
+        <v>4429.59333295</v>
       </c>
       <c r="H48" s="11" t="n">
         <f aca="false">G48+G47</f>
-        <v>4915.40857964235</v>
+        <v>4829.81057964235</v>
       </c>
       <c r="I48" s="11" t="n">
         <f aca="false">H48+H47</f>
-        <v>5493.07620480631</v>
+        <v>5241.21327080631</v>
       </c>
       <c r="J48" s="11" t="n">
         <f aca="false">I48+I47</f>
-        <v>6141.07620480631</v>
+        <v>5689.05198166229</v>
       </c>
       <c r="K48" s="11" t="n">
         <f aca="false">J48+J47</f>
-        <v>6843.07620480631</v>
+        <v>6246.88549889092</v>
       </c>
       <c r="L48" s="11" t="n">
         <f aca="false">K48+K47</f>
-        <v>7599.07620480631</v>
+        <v>6917.34417046523</v>
       </c>
       <c r="M48" s="11" t="n">
         <f aca="false">L48+L47</f>
-        <v>8413.57620480631</v>
+        <v>7686.88211104406</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5098,31 +5098,31 @@
       </c>
       <c r="G49" s="12" t="n">
         <f aca="false">Inputs!F25*(G48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.5769898901675</v>
+        <v>0.577067997359518</v>
       </c>
       <c r="H49" s="12" t="n">
         <f aca="false">Inputs!F25*(H48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.571093758188307</v>
+        <v>0.572097916338626</v>
       </c>
       <c r="I49" s="12" t="n">
         <f aca="false">Inputs!F25*(I48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.564783256848136</v>
+        <v>0.567440321178474</v>
       </c>
       <c r="J49" s="12" t="n">
         <f aca="false">Inputs!F25*(J48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.558520254441337</v>
+        <v>0.562806864258926</v>
       </c>
       <c r="K49" s="12" t="n">
         <f aca="false">Inputs!F25*(K48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.552507576972471</v>
+        <v>0.557566947957055</v>
       </c>
       <c r="L49" s="12" t="n">
         <f aca="false">Inputs!F25*(L48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.546748116851668</v>
+        <v>0.551911492377892</v>
       </c>
       <c r="M49" s="12" t="n">
         <f aca="false">Inputs!F25*(M48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.541209377011243</v>
+        <v>0.546120342338754</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5147,31 +5147,31 @@
       </c>
       <c r="G50" s="12" t="n">
         <f aca="false">F50*(1-Inputs!F29)+F52/MAX(F47,1)</f>
-        <v>0.933528549013727</v>
+        <v>0.933780596618873</v>
       </c>
       <c r="H50" s="12" t="n">
         <f aca="false">G50*(1-Inputs!F29)+G52/MAX(G47,1)</f>
-        <v>0.926863419470574</v>
+        <v>0.930425225265097</v>
       </c>
       <c r="I50" s="12" t="n">
         <f aca="false">H50*(1-Inputs!F29)+H52/MAX(H47,1)</f>
-        <v>0.919704502163673</v>
+        <v>0.929648647846222</v>
       </c>
       <c r="J50" s="12" t="n">
         <f aca="false">I50*(1-Inputs!F29)+I52/MAX(I47,1)</f>
-        <v>0.912336889609581</v>
+        <v>0.92901601763105</v>
       </c>
       <c r="K50" s="12" t="n">
         <f aca="false">J50*(1-Inputs!F29)+J52/MAX(J47,1)</f>
-        <v>0.904663795004669</v>
+        <v>0.924837518589791</v>
       </c>
       <c r="L50" s="12" t="n">
         <f aca="false">K50*(1-Inputs!F29)+K52/MAX(K47,1)</f>
-        <v>0.896349448806801</v>
+        <v>0.91784360002001</v>
       </c>
       <c r="M50" s="12" t="n">
         <f aca="false">L50*(1-Inputs!F29)+L52/MAX(L47,1)</f>
-        <v>0.887177360837091</v>
+        <v>0.908907540495577</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5288,35 +5288,35 @@
       </c>
       <c r="F53" s="10" t="n">
         <f aca="false">F50*F47</f>
-        <v>372.845896224325</v>
+        <v>367.20202040868</v>
       </c>
       <c r="G53" s="10" t="n">
         <f aca="false">G50*G47</f>
-        <v>447.921231039373</v>
+        <v>373.715099393545</v>
       </c>
       <c r="H53" s="10" t="n">
         <f aca="false">H50*H47</f>
-        <v>535.418990376916</v>
+        <v>382.779441600897</v>
       </c>
       <c r="I53" s="10" t="n">
         <f aca="false">I50*I47</f>
-        <v>595.96851740206</v>
+        <v>416.332652000454</v>
       </c>
       <c r="J53" s="10" t="n">
         <f aca="false">J50*J47</f>
-        <v>640.460496505926</v>
+        <v>518.23627267686</v>
       </c>
       <c r="K53" s="10" t="n">
         <f aca="false">K50*K47</f>
-        <v>683.92582902353</v>
+        <v>620.065334135792</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">L50*L47</f>
-        <v>730.076626053139</v>
+        <v>706.315473732858</v>
       </c>
       <c r="M53" s="10" t="n">
         <f aca="false">M50*M47</f>
-        <v>774.505836010781</v>
+        <v>759.827524596415</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5337,35 +5337,35 @@
       </c>
       <c r="F54" s="10" t="n">
         <f aca="false">F49*F47</f>
-        <v>230.853668945559</v>
+        <v>227.359170407936</v>
       </c>
       <c r="G54" s="10" t="n">
         <f aca="false">G49*G47</f>
-        <v>276.848546489711</v>
+        <v>230.952565057495</v>
       </c>
       <c r="H54" s="10" t="n">
         <f aca="false">H49*H47</f>
-        <v>329.902375038602</v>
+        <v>235.362622391006</v>
       </c>
       <c r="I54" s="10" t="n">
         <f aca="false">I49*I47</f>
-        <v>365.979550437592</v>
+        <v>254.121741924269</v>
       </c>
       <c r="J54" s="10" t="n">
         <f aca="false">J49*J47</f>
-        <v>392.081218617819</v>
+        <v>313.952532609971</v>
       </c>
       <c r="K54" s="10" t="n">
         <f aca="false">K49*K47</f>
-        <v>417.695728191188</v>
+        <v>373.825595241029</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">L49*L47</f>
-        <v>445.326341175683</v>
+        <v>424.716833226272</v>
       </c>
       <c r="M54" s="10" t="n">
         <f aca="false">M49*M47</f>
-        <v>472.475786130816</v>
+        <v>456.545082269588</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5386,35 +5386,35 @@
       </c>
       <c r="F55" s="10" t="n">
         <f aca="false">F53-F54-Inputs!E43-Decisions!F23</f>
-        <v>92.9922272787662</v>
+        <v>90.8428500007444</v>
       </c>
       <c r="G55" s="10" t="n">
         <f aca="false">G53-G54-Inputs!F43-Decisions!G23</f>
-        <v>118.072684549662</v>
+        <v>89.7625343360509</v>
       </c>
       <c r="H55" s="10" t="n">
         <f aca="false">H53-H54-Inputs!G43-Decisions!H23</f>
-        <v>148.516615338315</v>
+        <v>90.4168192098907</v>
       </c>
       <c r="I55" s="10" t="n">
         <f aca="false">I53-I54-Inputs!H43-Decisions!I23</f>
-        <v>168.988966964468</v>
+        <v>101.210910076185</v>
       </c>
       <c r="J55" s="10" t="n">
         <f aca="false">J53-J54-Inputs!I43-Decisions!J23</f>
-        <v>183.379277888107</v>
+        <v>139.28374006689</v>
       </c>
       <c r="K55" s="10" t="n">
         <f aca="false">K53-K54-Inputs!J43-Decisions!K23</f>
-        <v>197.230100832342</v>
+        <v>177.239738894763</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">L53-L54-Inputs!K43-Decisions!L23</f>
-        <v>211.750284877456</v>
+        <v>208.598640506586</v>
       </c>
       <c r="M55" s="10" t="n">
         <f aca="false">M53-M54-Inputs!L43-Decisions!M23</f>
-        <v>225.030049879965</v>
+        <v>226.282442326827</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5446,27 +5446,27 @@
       </c>
       <c r="H57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*G57+(Decisions!D16)/Inputs!G22</f>
-        <v>11.2221979724254</v>
+        <v>11.0555313057587</v>
       </c>
       <c r="I57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*H57+(Decisions!E16)/Inputs!G22</f>
-        <v>12.5536440416062</v>
+        <v>11.0648107082729</v>
       </c>
       <c r="J57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*I57+(Decisions!F16)/Inputs!G22</f>
-        <v>14.6292165574853</v>
+        <v>11.1568017241519</v>
       </c>
       <c r="K57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*J57+(Decisions!G16)/Inputs!G22</f>
-        <v>16.5657257148004</v>
+        <v>11.7426293419671</v>
       </c>
       <c r="L57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*K57+(Decisions!H16)/Inputs!G22</f>
-        <v>18.7891554252421</v>
+        <v>13.9558731760553</v>
       </c>
       <c r="M57" s="10" t="n">
         <f aca="false">(1-Inputs!G24)*L57+(Decisions!I16)/Inputs!G22</f>
-        <v>20.4469486784176</v>
+        <v>16.3541630065929</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5495,27 +5495,27 @@
       </c>
       <c r="H58" s="10" t="n">
         <f aca="false">MIN(H57,Inputs!G21*Decisions!H8)</f>
-        <v>11.2221979724254</v>
+        <v>11.0555313057587</v>
       </c>
       <c r="I58" s="10" t="n">
         <f aca="false">MIN(I57,Inputs!G21*Decisions!I8)</f>
-        <v>12.5536440416062</v>
+        <v>11.0648107082729</v>
       </c>
       <c r="J58" s="10" t="n">
         <f aca="false">MIN(J57,Inputs!G21*Decisions!J8)</f>
-        <v>14.6292165574853</v>
+        <v>11.1568017241519</v>
       </c>
       <c r="K58" s="10" t="n">
         <f aca="false">MIN(K57,Inputs!G21*Decisions!K8)</f>
-        <v>16.5657257148004</v>
+        <v>11.7426293419671</v>
       </c>
       <c r="L58" s="10" t="n">
         <f aca="false">MIN(L57,Inputs!G21*Decisions!L8)</f>
-        <v>18.7891554252421</v>
+        <v>13.9558731760553</v>
       </c>
       <c r="M58" s="10" t="n">
         <f aca="false">MIN(M57,Inputs!G21*Decisions!M8)</f>
-        <v>20.4469486784176</v>
+        <v>16.3541630065929</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5548,23 +5548,23 @@
       </c>
       <c r="I59" s="11" t="n">
         <f aca="false">H59+H58</f>
-        <v>115.119740672544</v>
+        <v>114.953074005877</v>
       </c>
       <c r="J59" s="11" t="n">
         <f aca="false">I59+I58</f>
-        <v>127.67338471415</v>
+        <v>126.01788471415</v>
       </c>
       <c r="K59" s="11" t="n">
         <f aca="false">J59+J58</f>
-        <v>142.302601271636</v>
+        <v>137.174686438302</v>
       </c>
       <c r="L59" s="11" t="n">
         <f aca="false">K59+K58</f>
-        <v>158.868326986436</v>
+        <v>148.917315780269</v>
       </c>
       <c r="M59" s="11" t="n">
         <f aca="false">L59+L58</f>
-        <v>177.657482411678</v>
+        <v>162.873188956325</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5597,23 +5597,23 @@
       </c>
       <c r="I60" s="12" t="n">
         <f aca="false">Inputs!G25*(I59/Inputs!G27)^(-Inputs!G26)</f>
-        <v>3.87275613043626</v>
+        <v>3.87376622678499</v>
       </c>
       <c r="J60" s="12" t="n">
         <f aca="false">Inputs!G25*(J59/Inputs!G27)^(-Inputs!G26)</f>
-        <v>3.8012728835183</v>
+        <v>3.81021358538508</v>
       </c>
       <c r="K60" s="12" t="n">
         <f aca="false">Inputs!G25*(K59/Inputs!G27)^(-Inputs!G26)</f>
-        <v>3.72776737859604</v>
+        <v>3.75247492494635</v>
       </c>
       <c r="L60" s="12" t="n">
         <f aca="false">Inputs!G25*(L59/Inputs!G27)^(-Inputs!G26)</f>
-        <v>3.65460460045225</v>
+        <v>3.69740461232113</v>
       </c>
       <c r="M60" s="12" t="n">
         <f aca="false">Inputs!G25*(M59/Inputs!G27)^(-Inputs!G26)</f>
-        <v>3.58180620055777</v>
+        <v>3.63826381094495</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5646,23 +5646,23 @@
       </c>
       <c r="I61" s="12" t="n">
         <f aca="false">H61*(1-Inputs!G29)+H63/MAX(H58,1)</f>
-        <v>6.88317323100192</v>
+        <v>6.89274464438892</v>
       </c>
       <c r="J61" s="12" t="n">
         <f aca="false">I61*(1-Inputs!G29)+I63/MAX(I58,1)</f>
-        <v>7.62542428065923</v>
+        <v>7.73945279631801</v>
       </c>
       <c r="K61" s="12" t="n">
         <f aca="false">J61*(1-Inputs!G29)+J63/MAX(J58,1)</f>
-        <v>8.63827620106478</v>
+        <v>9.07883864075239</v>
       </c>
       <c r="L61" s="12" t="n">
         <f aca="false">K61*(1-Inputs!G29)+K63/MAX(K58,1)</f>
-        <v>9.86276245528903</v>
+        <v>10.8218003079306</v>
       </c>
       <c r="M61" s="12" t="n">
         <f aca="false">L61*(1-Inputs!G29)+L63/MAX(L58,1)</f>
-        <v>11.1945644735378</v>
+        <v>12.6271235090655</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5785,27 +5785,27 @@
       </c>
       <c r="H64" s="10" t="n">
         <f aca="false">H61*H58</f>
-        <v>70.4716911324647</v>
+        <v>69.4250795966256</v>
       </c>
       <c r="I64" s="10" t="n">
         <f aca="false">I61*I58</f>
-        <v>86.4089066187107</v>
+        <v>76.2669147506252</v>
       </c>
       <c r="J64" s="10" t="n">
         <f aca="false">J61*J58</f>
-        <v>111.55398314447</v>
+        <v>86.3475403019533</v>
       </c>
       <c r="K64" s="10" t="n">
         <f aca="false">K61*K58</f>
-        <v>143.099314195527</v>
+        <v>106.609437013884</v>
       </c>
       <c r="L64" s="10" t="n">
         <f aca="false">L61*L58</f>
-        <v>185.312976694668</v>
+        <v>151.027672634075</v>
       </c>
       <c r="M64" s="10" t="n">
         <f aca="false">M61*M58</f>
-        <v>228.894685267663</v>
+        <v>206.50603617164</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5834,27 +5834,27 @@
       </c>
       <c r="H65" s="10" t="n">
         <f aca="false">H60*H58</f>
-        <v>44.2706695951366</v>
+        <v>43.6131829823846</v>
       </c>
       <c r="I65" s="10" t="n">
         <f aca="false">I60*I58</f>
-        <v>48.6172019214451</v>
+        <v>42.8624900274765</v>
       </c>
       <c r="J65" s="10" t="n">
         <f aca="false">J60*J58</f>
-        <v>55.6096442070857</v>
+        <v>42.5097974988114</v>
       </c>
       <c r="K65" s="10" t="n">
         <f aca="false">K60*K58</f>
-        <v>61.7531719224026</v>
+        <v>44.0639221586708</v>
       </c>
       <c r="L65" s="10" t="n">
         <f aca="false">L60*L58</f>
-        <v>68.6669338557023</v>
+        <v>51.6005098501155</v>
       </c>
       <c r="M65" s="10" t="n">
         <f aca="false">M60*M58</f>
-        <v>73.2370075588426</v>
+        <v>59.5007594251818</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5883,27 +5883,27 @@
       </c>
       <c r="H66" s="10" t="n">
         <f aca="false">H64-H65-Inputs!G44-Decisions!H24</f>
-        <v>-10.7989784626719</v>
+        <v>-11.188103385759</v>
       </c>
       <c r="I66" s="10" t="n">
         <f aca="false">I64-I65-Inputs!H44-Decisions!I24</f>
-        <v>-3.20829530273441</v>
+        <v>-7.59557527685132</v>
       </c>
       <c r="J66" s="10" t="n">
         <f aca="false">J64-J65-Inputs!I44-Decisions!J24</f>
-        <v>10.9443389373844</v>
+        <v>-1.16225719685809</v>
       </c>
       <c r="K66" s="10" t="n">
         <f aca="false">K64-K65-Inputs!J44-Decisions!K24</f>
-        <v>32.3461422731247</v>
+        <v>13.5455148552129</v>
       </c>
       <c r="L66" s="10" t="n">
         <f aca="false">L64-L65-Inputs!K44-Decisions!L24</f>
-        <v>63.646042838966</v>
+        <v>46.4271627839599</v>
       </c>
       <c r="M66" s="10" t="n">
         <f aca="false">M64-M65-Inputs!L44-Decisions!M24</f>
-        <v>98.6576777088208</v>
+        <v>90.0052767464579</v>
       </c>
     </row>
   </sheetData>
@@ -5989,31 +5989,31 @@
       </c>
       <c r="F2" s="13" t="n">
         <f aca="false">Dynamics!G11</f>
-        <v>-1.24898048013472</v>
+        <v>-1.38901270864005</v>
       </c>
       <c r="G2" s="13" t="n">
         <f aca="false">Dynamics!H11</f>
-        <v>0.640091749889621</v>
+        <v>-1.3546278918617</v>
       </c>
       <c r="H2" s="13" t="n">
         <f aca="false">Dynamics!I11</f>
-        <v>4.06226678766274</v>
+        <v>-0.212673566792859</v>
       </c>
       <c r="I2" s="13" t="n">
         <f aca="false">Dynamics!J11</f>
-        <v>13.5973828031006</v>
+        <v>6.80821201680257</v>
       </c>
       <c r="J2" s="13" t="n">
         <f aca="false">Dynamics!K11</f>
-        <v>26.5117810565617</v>
+        <v>20.2554323496811</v>
       </c>
       <c r="K2" s="13" t="n">
         <f aca="false">Dynamics!L11</f>
-        <v>42.2596881267166</v>
+        <v>37.4804104390084</v>
       </c>
       <c r="L2" s="13" t="n">
         <f aca="false">Dynamics!M11</f>
-        <v>59.64358455473</v>
+        <v>57.4070422942264</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6030,39 +6030,39 @@
       </c>
       <c r="D3" s="13" t="n">
         <f aca="false">Dynamics!E22</f>
-        <v>15.8531476766989</v>
+        <v>15.0723744473576</v>
       </c>
       <c r="E3" s="13" t="n">
         <f aca="false">Dynamics!F22</f>
-        <v>30.8773086564933</v>
+        <v>19.1562215538352</v>
       </c>
       <c r="F3" s="13" t="n">
         <f aca="false">Dynamics!G22</f>
-        <v>61.5205786586931</v>
+        <v>34.6134631954567</v>
       </c>
       <c r="G3" s="13" t="n">
         <f aca="false">Dynamics!H22</f>
-        <v>110.53391043471</v>
+        <v>67.5205996763273</v>
       </c>
       <c r="H3" s="13" t="n">
         <f aca="false">Dynamics!I22</f>
-        <v>168.331274938205</v>
+        <v>135.133052010671</v>
       </c>
       <c r="I3" s="13" t="n">
         <f aca="false">Dynamics!J22</f>
-        <v>235.058311133993</v>
+        <v>218.008811679595</v>
       </c>
       <c r="J3" s="13" t="n">
         <f aca="false">Dynamics!K22</f>
-        <v>294.406278237303</v>
+        <v>303.148838462092</v>
       </c>
       <c r="K3" s="13" t="n">
         <f aca="false">Dynamics!L22</f>
-        <v>347.874025602136</v>
+        <v>378.514716973411</v>
       </c>
       <c r="L3" s="13" t="n">
         <f aca="false">Dynamics!M22</f>
-        <v>392.360577261666</v>
+        <v>439.66394698948</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6083,35 +6083,35 @@
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">Dynamics!F33</f>
-        <v>-11.3801623422023</v>
+        <v>-11.453533526154</v>
       </c>
       <c r="F4" s="13" t="n">
         <f aca="false">Dynamics!G33</f>
-        <v>-10.9481524790998</v>
+        <v>-12.4789578192194</v>
       </c>
       <c r="G4" s="13" t="n">
         <f aca="false">Dynamics!H33</f>
-        <v>-9.0082768655934</v>
+        <v>-12.6635243126684</v>
       </c>
       <c r="H4" s="13" t="n">
         <f aca="false">Dynamics!I33</f>
-        <v>-5.42892527297296</v>
+        <v>-11.2504095181181</v>
       </c>
       <c r="I4" s="13" t="n">
         <f aca="false">Dynamics!J33</f>
-        <v>2.44635228909446</v>
+        <v>-2.61464869872807</v>
       </c>
       <c r="J4" s="13" t="n">
         <f aca="false">Dynamics!K33</f>
-        <v>13.0332752142127</v>
+        <v>10.4568147054286</v>
       </c>
       <c r="K4" s="13" t="n">
         <f aca="false">Dynamics!L33</f>
-        <v>25.6871506252367</v>
+        <v>27.0154152389962</v>
       </c>
       <c r="L4" s="13" t="n">
         <f aca="false">Dynamics!M33</f>
-        <v>39.6889600345054</v>
+        <v>44.8299480370181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6136,31 +6136,31 @@
       </c>
       <c r="F5" s="13" t="n">
         <f aca="false">Dynamics!G44</f>
-        <v>-26.005097448887</v>
+        <v>-26.226935252054</v>
       </c>
       <c r="G5" s="13" t="n">
         <f aca="false">Dynamics!H44</f>
-        <v>-19.5059014463545</v>
+        <v>-23.556866405409</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">Dynamics!I44</f>
-        <v>-6.32621867480042</v>
+        <v>-17.1211868352275</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">Dynamics!J44</f>
-        <v>14.4344251780161</v>
+        <v>-3.78760526461738</v>
       </c>
       <c r="J5" s="13" t="n">
         <f aca="false">Dynamics!K44</f>
-        <v>45.225770761512</v>
+        <v>33.2338788323841</v>
       </c>
       <c r="K5" s="13" t="n">
         <f aca="false">Dynamics!L44</f>
-        <v>84.6268872950972</v>
+        <v>87.5632188532965</v>
       </c>
       <c r="L5" s="13" t="n">
         <f aca="false">Dynamics!M44</f>
-        <v>128.713545634631</v>
+        <v>151.716877146872</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6181,35 +6181,35 @@
       </c>
       <c r="E6" s="13" t="n">
         <f aca="false">Dynamics!F55</f>
-        <v>92.9922272787662</v>
+        <v>90.8428500007444</v>
       </c>
       <c r="F6" s="13" t="n">
         <f aca="false">Dynamics!G55</f>
-        <v>118.072684549662</v>
+        <v>89.7625343360509</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">Dynamics!H55</f>
-        <v>148.516615338315</v>
+        <v>90.4168192098907</v>
       </c>
       <c r="H6" s="13" t="n">
         <f aca="false">Dynamics!I55</f>
-        <v>168.988966964468</v>
+        <v>101.210910076185</v>
       </c>
       <c r="I6" s="13" t="n">
         <f aca="false">Dynamics!J55</f>
-        <v>183.379277888107</v>
+        <v>139.28374006689</v>
       </c>
       <c r="J6" s="13" t="n">
         <f aca="false">Dynamics!K55</f>
-        <v>197.230100832342</v>
+        <v>177.239738894763</v>
       </c>
       <c r="K6" s="13" t="n">
         <f aca="false">Dynamics!L55</f>
-        <v>211.750284877456</v>
+        <v>208.598640506586</v>
       </c>
       <c r="L6" s="13" t="n">
         <f aca="false">Dynamics!M55</f>
-        <v>225.030049879965</v>
+        <v>226.282442326827</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6238,27 +6238,27 @@
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">Dynamics!H66</f>
-        <v>-10.7989784626719</v>
+        <v>-11.188103385759</v>
       </c>
       <c r="H7" s="13" t="n">
         <f aca="false">Dynamics!I66</f>
-        <v>-3.20829530273441</v>
+        <v>-7.59557527685132</v>
       </c>
       <c r="I7" s="13" t="n">
         <f aca="false">Dynamics!J66</f>
-        <v>10.9443389373844</v>
+        <v>-1.16225719685809</v>
       </c>
       <c r="J7" s="13" t="n">
         <f aca="false">Dynamics!K66</f>
-        <v>32.3461422731247</v>
+        <v>13.5455148552129</v>
       </c>
       <c r="K7" s="13" t="n">
         <f aca="false">Dynamics!L66</f>
-        <v>63.646042838966</v>
+        <v>46.4271627839599</v>
       </c>
       <c r="L7" s="13" t="n">
         <f aca="false">Dynamics!M66</f>
-        <v>98.6576777088208</v>
+        <v>90.0052767464579</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6275,39 +6275,39 @@
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">SUM(D2:D7)</f>
-        <v>69.3293625480451</v>
+        <v>68.5485893187038</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">SUM(E2:E7)</f>
-        <v>75.6959919687453</v>
+        <v>61.7521564041138</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">SUM(F2:F7)</f>
-        <v>127.933988224483</v>
+        <v>70.8240471758434</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">SUM(G2:G7)</f>
-        <v>220.377460748294</v>
+        <v>109.17429689052</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">SUM(H2:H7)</f>
-        <v>326.419069439827</v>
+        <v>200.164116889866</v>
       </c>
       <c r="I8" s="14" t="n">
         <f aca="false">SUM(I2:I7)</f>
-        <v>459.860088229695</v>
+        <v>356.536252603083</v>
       </c>
       <c r="J8" s="14" t="n">
         <f aca="false">SUM(J2:J7)</f>
-        <v>608.753348375056</v>
+        <v>557.880218099562</v>
       </c>
       <c r="K8" s="14" t="n">
         <f aca="false">SUM(K2:K7)</f>
-        <v>775.844079365609</v>
+        <v>785.599564795258</v>
       </c>
       <c r="L8" s="14" t="n">
         <f aca="false">SUM(L2:L7)</f>
-        <v>944.094395074319</v>
+        <v>1009.90553354088</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6324,39 +6324,39 @@
       </c>
       <c r="D9" s="14" t="n">
         <f aca="false">Dynamics!E9+Dynamics!E20+Dynamics!E31+Dynamics!E42+Dynamics!E53+Dynamics!E64</f>
-        <v>1107.35208580455</v>
+        <v>1104.44141080455</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">Dynamics!F9+Dynamics!F20+Dynamics!F31+Dynamics!F42+Dynamics!F53+Dynamics!F64</f>
-        <v>1152.06913273106</v>
+        <v>1106.15955344684</v>
       </c>
       <c r="F9" s="14" t="n">
         <f aca="false">Dynamics!G9+Dynamics!G20+Dynamics!G31+Dynamics!G42+Dynamics!G53+Dynamics!G64</f>
-        <v>1288.64547072509</v>
+        <v>1123.60913846944</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">Dynamics!H9+Dynamics!H20+Dynamics!H31+Dynamics!H42+Dynamics!H53+Dynamics!H64</f>
-        <v>1488.85472483581</v>
+        <v>1179.89371439247</v>
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">Dynamics!I9+Dynamics!I20+Dynamics!I31+Dynamics!I42+Dynamics!I53+Dynamics!I64</f>
-        <v>1684.50272863087</v>
+        <v>1327.80652128725</v>
       </c>
       <c r="I9" s="14" t="n">
         <f aca="false">Dynamics!J9+Dynamics!J20+Dynamics!J31+Dynamics!J42+Dynamics!J53+Dynamics!J64</f>
-        <v>1901.66546156845</v>
+        <v>1594.60386687797</v>
       </c>
       <c r="J9" s="14" t="n">
         <f aca="false">Dynamics!K9+Dynamics!K20+Dynamics!K31+Dynamics!K42+Dynamics!K53+Dynamics!K64</f>
-        <v>2116.81163620404</v>
+        <v>1914.24728872847</v>
       </c>
       <c r="K9" s="14" t="n">
         <f aca="false">Dynamics!L9+Dynamics!L20+Dynamics!L31+Dynamics!L42+Dynamics!L53+Dynamics!L64</f>
-        <v>2343.63056699885</v>
+        <v>2248.20936431734</v>
       </c>
       <c r="L9" s="14" t="n">
         <f aca="false">Dynamics!M9+Dynamics!M20+Dynamics!M31+Dynamics!M42+Dynamics!M53+Dynamics!M64</f>
-        <v>2560.67958532693</v>
+        <v>2549.25025422893</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6369,43 +6369,43 @@
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">Decisions!D11+Decisions!D12+Decisions!D13+Decisions!D14+Decisions!D15+Decisions!D16</f>
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">Decisions!E11+Decisions!E12+Decisions!E13+Decisions!E14+Decisions!E15+Decisions!E16</f>
-        <v>220</v>
+        <v>70</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">Decisions!F11+Decisions!F12+Decisions!F13+Decisions!F14+Decisions!F15+Decisions!F16</f>
-        <v>260</v>
+        <v>75</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">Decisions!G11+Decisions!G12+Decisions!G13+Decisions!G14+Decisions!G15+Decisions!G16</f>
-        <v>295</v>
+        <v>125</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">Decisions!H11+Decisions!H12+Decisions!H13+Decisions!H14+Decisions!H15+Decisions!H16</f>
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">Decisions!I11+Decisions!I12+Decisions!I13+Decisions!I14+Decisions!I15+Decisions!I16</f>
-        <v>250</v>
+        <v>295</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">Decisions!J11+Decisions!J12+Decisions!J13+Decisions!J14+Decisions!J15+Decisions!J16</f>
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="J10" s="10" t="n">
         <f aca="false">Decisions!K11+Decisions!K12+Decisions!K13+Decisions!K14+Decisions!K15+Decisions!K16</f>
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">Decisions!L11+Decisions!L12+Decisions!L13+Decisions!L14+Decisions!L15+Decisions!L16</f>
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">Decisions!M11+Decisions!M12+Decisions!M13+Decisions!M14+Decisions!M15+Decisions!M16</f>
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6467,43 +6467,43 @@
       </c>
       <c r="C12" s="14" t="n">
         <f aca="false">C8*(1-Inputs!B3)+Inputs!B3*C11-C10</f>
-        <v>-14.6243023168091</v>
+        <v>-1.62430231680906</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">D8*(1-Inputs!B3)+Inputs!B3*D11-D10</f>
-        <v>-150.489565339927</v>
+        <v>-1.05952979734622</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">E8*(1-Inputs!B3)+Inputs!B3*E11-E10</f>
-        <v>-183.681925862816</v>
+        <v>-8.86092582499694</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">F8*(1-Inputs!B3)+Inputs!B3*F11-F10</f>
-        <v>-177.848188596128</v>
+        <v>-49.5384455616343</v>
       </c>
       <c r="G12" s="14" t="n">
         <f aca="false">G8*(1-Inputs!B3)+Inputs!B3*G11-G10</f>
-        <v>-92.1244536537454</v>
+        <v>-168.302763269921</v>
       </c>
       <c r="H12" s="14" t="n">
         <f aca="false">H8*(1-Inputs!B3)+Inputs!B3*H11-H10</f>
-        <v>19.3359206910738</v>
+        <v>-117.830194670398</v>
       </c>
       <c r="I12" s="14" t="n">
         <f aca="false">I8*(1-Inputs!B3)+Inputs!B3*I11-I10</f>
-        <v>160.797864407678</v>
+        <v>15.3714644002508</v>
       </c>
       <c r="J12" s="14" t="n">
         <f aca="false">J8*(1-Inputs!B3)+Inputs!B3*J11-J10</f>
-        <v>314.889944313791</v>
+        <v>217.75255921268</v>
       </c>
       <c r="K12" s="14" t="n">
         <f aca="false">K8*(1-Inputs!B3)+Inputs!B3*K11-K10</f>
-        <v>474.266177936894</v>
+        <v>439.387682300538</v>
       </c>
       <c r="L12" s="14" t="n">
         <f aca="false">L8*(1-Inputs!B3)+Inputs!B3*L11-L10</f>
-        <v>631.838908404253</v>
+        <v>669.881039484843</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6582,43 +6582,43 @@
       </c>
       <c r="C18" s="10" t="n">
         <f aca="false">C12*C17</f>
-        <v>-13.3567470242114</v>
+        <v>-1.48351659220848</v>
       </c>
       <c r="D18" s="10" t="n">
         <f aca="false">D12*D17</f>
-        <v>-125.532875281404</v>
+        <v>-0.883820892211089</v>
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">E12*E17</f>
-        <v>-139.940382589076</v>
+        <v>-6.75080764870465</v>
       </c>
       <c r="F18" s="10" t="n">
         <f aca="false">F12*F17</f>
-        <v>-123.751828085096</v>
+        <v>-34.4702594225902</v>
       </c>
       <c r="G18" s="10" t="n">
         <f aca="false">G12*G17</f>
-        <v>-58.5467303942668</v>
+        <v>-106.959402362475</v>
       </c>
       <c r="H18" s="10" t="n">
         <f aca="false">H12*H17</f>
-        <v>11.2232366771049</v>
+        <v>-68.3927175552442</v>
       </c>
       <c r="I18" s="10" t="n">
         <f aca="false">I12*I17</f>
-        <v>85.2430707494901</v>
+        <v>8.14880740002715</v>
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">J12*J17</f>
-        <v>152.46253831368</v>
+        <v>105.430829092408</v>
       </c>
       <c r="K18" s="10" t="n">
         <f aca="false">K12*K17</f>
-        <v>209.725893032427</v>
+        <v>194.302225933113</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">L12*L17</f>
-        <v>255.188916763794</v>
+        <v>270.553482150184</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">L12*(1+Inputs!B9)</f>
-        <v>647.634881114359</v>
+        <v>686.628065471964</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="B22" s="14" t="n">
         <f aca="false">B21/($B$15-Inputs!B9)</f>
-        <v>9265.16281994792</v>
+        <v>9823.00522849734</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">B22*L17</f>
-        <v>3742.04062493404</v>
+        <v>3967.34362237394</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="B25" s="19" t="n">
         <f aca="false">SUM(C18:L18)</f>
-        <v>252.715092162442</v>
+        <v>359.494820102299</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">B25+B23</f>
-        <v>3994.75571709648</v>
+        <v>4326.83844247624</v>
       </c>
     </row>
   </sheetData>
@@ -6848,39 +6848,39 @@
       </c>
       <c r="D4" s="13" t="n">
         <f aca="false">Financials!D9</f>
-        <v>1107.35208580455</v>
+        <v>1104.44141080455</v>
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">Financials!E9</f>
-        <v>1152.06913273106</v>
+        <v>1106.15955344684</v>
       </c>
       <c r="F4" s="13" t="n">
         <f aca="false">Financials!F9</f>
-        <v>1288.64547072509</v>
+        <v>1123.60913846944</v>
       </c>
       <c r="G4" s="13" t="n">
         <f aca="false">Financials!G9</f>
-        <v>1488.85472483581</v>
+        <v>1179.89371439247</v>
       </c>
       <c r="H4" s="13" t="n">
         <f aca="false">Financials!H9</f>
-        <v>1684.50272863087</v>
+        <v>1327.80652128725</v>
       </c>
       <c r="I4" s="13" t="n">
         <f aca="false">Financials!I9</f>
-        <v>1901.66546156845</v>
+        <v>1594.60386687797</v>
       </c>
       <c r="J4" s="13" t="n">
         <f aca="false">Financials!J9</f>
-        <v>2116.81163620404</v>
+        <v>1914.24728872847</v>
       </c>
       <c r="K4" s="13" t="n">
         <f aca="false">Financials!K9</f>
-        <v>2343.63056699885</v>
+        <v>2248.20936431734</v>
       </c>
       <c r="L4" s="13" t="n">
         <f aca="false">Financials!L9</f>
-        <v>2560.67958532693</v>
+        <v>2549.25025422893</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6897,39 +6897,39 @@
       </c>
       <c r="D5" s="13" t="n">
         <f aca="false">Financials!D8</f>
-        <v>69.3293625480451</v>
+        <v>68.5485893187038</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">Financials!E8</f>
-        <v>75.6959919687453</v>
+        <v>61.7521564041138</v>
       </c>
       <c r="F5" s="13" t="n">
         <f aca="false">Financials!F8</f>
-        <v>127.933988224483</v>
+        <v>70.8240471758434</v>
       </c>
       <c r="G5" s="13" t="n">
         <f aca="false">Financials!G8</f>
-        <v>220.377460748294</v>
+        <v>109.17429689052</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">Financials!H8</f>
-        <v>326.419069439827</v>
+        <v>200.164116889866</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">Financials!I8</f>
-        <v>459.860088229695</v>
+        <v>356.536252603083</v>
       </c>
       <c r="J5" s="13" t="n">
         <f aca="false">Financials!J8</f>
-        <v>608.753348375056</v>
+        <v>557.880218099562</v>
       </c>
       <c r="K5" s="13" t="n">
         <f aca="false">Financials!K8</f>
-        <v>775.844079365609</v>
+        <v>785.599564795258</v>
       </c>
       <c r="L5" s="13" t="n">
         <f aca="false">Financials!L8</f>
-        <v>944.094395074319</v>
+        <v>1009.90553354088</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6991,43 +6991,43 @@
       </c>
       <c r="C7" s="13" t="n">
         <f aca="false">Financials!C10</f>
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="D7" s="13" t="n">
         <f aca="false">Financials!D10</f>
-        <v>220</v>
+        <v>70</v>
       </c>
       <c r="E7" s="13" t="n">
         <f aca="false">Financials!E10</f>
-        <v>260</v>
+        <v>75</v>
       </c>
       <c r="F7" s="13" t="n">
         <f aca="false">Financials!F10</f>
-        <v>295</v>
+        <v>125</v>
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">Financials!G10</f>
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="H7" s="13" t="n">
         <f aca="false">Financials!H10</f>
-        <v>250</v>
+        <v>295</v>
       </c>
       <c r="I7" s="13" t="n">
         <f aca="false">Financials!I10</f>
-        <v>210</v>
+        <v>280</v>
       </c>
       <c r="J7" s="13" t="n">
         <f aca="false">Financials!J10</f>
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="K7" s="13" t="n">
         <f aca="false">Financials!K10</f>
-        <v>138</v>
+        <v>180</v>
       </c>
       <c r="L7" s="13" t="n">
         <f aca="false">Financials!L10</f>
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7040,43 +7040,43 @@
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">Financials!C12</f>
-        <v>-14.6243023168091</v>
+        <v>-1.62430231680906</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">Financials!D12</f>
-        <v>-150.489565339927</v>
+        <v>-1.05952979734622</v>
       </c>
       <c r="E8" s="13" t="n">
         <f aca="false">Financials!E12</f>
-        <v>-183.681925862816</v>
+        <v>-8.86092582499694</v>
       </c>
       <c r="F8" s="13" t="n">
         <f aca="false">Financials!F12</f>
-        <v>-177.848188596128</v>
+        <v>-49.5384455616343</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">Financials!G12</f>
-        <v>-92.1244536537454</v>
+        <v>-168.302763269921</v>
       </c>
       <c r="H8" s="13" t="n">
         <f aca="false">Financials!H12</f>
-        <v>19.3359206910738</v>
+        <v>-117.830194670398</v>
       </c>
       <c r="I8" s="13" t="n">
         <f aca="false">Financials!I12</f>
-        <v>160.797864407678</v>
+        <v>15.3714644002508</v>
       </c>
       <c r="J8" s="13" t="n">
         <f aca="false">Financials!J12</f>
-        <v>314.889944313791</v>
+        <v>217.75255921268</v>
       </c>
       <c r="K8" s="13" t="n">
         <f aca="false">Financials!K12</f>
-        <v>474.266177936894</v>
+        <v>439.387682300538</v>
       </c>
       <c r="L8" s="13" t="n">
         <f aca="false">Financials!L12</f>
-        <v>631.838908404253</v>
+        <v>669.881039484843</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7138,43 +7138,43 @@
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">Financials!C18</f>
-        <v>-13.3567470242114</v>
+        <v>-1.48351659220848</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">Financials!D18</f>
-        <v>-125.532875281404</v>
+        <v>-0.883820892211089</v>
       </c>
       <c r="E10" s="13" t="n">
         <f aca="false">Financials!E18</f>
-        <v>-139.940382589076</v>
+        <v>-6.75080764870465</v>
       </c>
       <c r="F10" s="13" t="n">
         <f aca="false">Financials!F18</f>
-        <v>-123.751828085096</v>
+        <v>-34.4702594225902</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">Financials!G18</f>
-        <v>-58.5467303942668</v>
+        <v>-106.959402362475</v>
       </c>
       <c r="H10" s="13" t="n">
         <f aca="false">Financials!H18</f>
-        <v>11.2232366771049</v>
+        <v>-68.3927175552442</v>
       </c>
       <c r="I10" s="13" t="n">
         <f aca="false">Financials!I18</f>
-        <v>85.2430707494901</v>
+        <v>8.14880740002715</v>
       </c>
       <c r="J10" s="13" t="n">
         <f aca="false">Financials!J18</f>
-        <v>152.46253831368</v>
+        <v>105.430829092408</v>
       </c>
       <c r="K10" s="13" t="n">
         <f aca="false">Financials!K18</f>
-        <v>209.725893032427</v>
+        <v>194.302225933113</v>
       </c>
       <c r="L10" s="13" t="n">
         <f aca="false">Financials!L18</f>
-        <v>255.188916763794</v>
+        <v>270.553482150184</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7204,31 +7204,31 @@
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">Dynamics!G9</f>
-        <v>361.307637833258</v>
+        <v>360.57172563799</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">Dynamics!H9</f>
-        <v>355.347654753688</v>
+        <v>345.935458189399</v>
       </c>
       <c r="H13" s="13" t="n">
         <f aca="false">Dynamics!I9</f>
-        <v>353.080259269405</v>
+        <v>334.43924283803</v>
       </c>
       <c r="I13" s="13" t="n">
         <f aca="false">Dynamics!J9</f>
-        <v>359.796342174353</v>
+        <v>332.521746962887</v>
       </c>
       <c r="J13" s="13" t="n">
         <f aca="false">Dynamics!K9</f>
-        <v>369.59258218974</v>
+        <v>344.540181880773</v>
       </c>
       <c r="K13" s="13" t="n">
         <f aca="false">Dynamics!L9</f>
-        <v>381.943273497876</v>
+        <v>361.416157175286</v>
       </c>
       <c r="L13" s="13" t="n">
         <f aca="false">Dynamics!M9</f>
-        <v>394.729661955163</v>
+        <v>380.83717058262</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7245,39 +7245,39 @@
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">Dynamics!E20</f>
-        <v>197.0333124045</v>
+        <v>194.1226374045</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">Dynamics!F20</f>
-        <v>240.183750465257</v>
+        <v>200.294523796682</v>
       </c>
       <c r="F14" s="13" t="n">
         <f aca="false">Dynamics!G20</f>
-        <v>302.421634855314</v>
+        <v>220.001838246704</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">Dynamics!H20</f>
-        <v>385.120937746048</v>
+        <v>264.316198533048</v>
       </c>
       <c r="H14" s="13" t="n">
         <f aca="false">Dynamics!I20</f>
-        <v>468.361266950262</v>
+        <v>364.875858463511</v>
       </c>
       <c r="I14" s="13" t="n">
         <f aca="false">Dynamics!J20</f>
-        <v>558.241835751447</v>
+        <v>480.772725931765</v>
       </c>
       <c r="J14" s="13" t="n">
         <f aca="false">Dynamics!K20</f>
-        <v>629.030648333135</v>
+        <v>592.989054410623</v>
       </c>
       <c r="K14" s="13" t="n">
         <f aca="false">Dynamics!L20</f>
-        <v>688.438599146845</v>
+        <v>686.240326573857</v>
       </c>
       <c r="L14" s="13" t="n">
         <f aca="false">Dynamics!M20</f>
-        <v>733.99347611162</v>
+        <v>757.143582306482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7298,35 +7298,35 @@
       </c>
       <c r="E15" s="13" t="n">
         <f aca="false">Dynamics!F31</f>
-        <v>69.8851050475603</v>
+        <v>69.5086282475603</v>
       </c>
       <c r="F15" s="13" t="n">
         <f aca="false">Dynamics!G31</f>
-        <v>76.3254597083408</v>
+        <v>69.4350875028964</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">Dynamics!H31</f>
-        <v>85.4470842464502</v>
+        <v>70.4167371477603</v>
       </c>
       <c r="H15" s="13" t="n">
         <f aca="false">Dynamics!I31</f>
-        <v>97.2442643462017</v>
+        <v>74.9307990636234</v>
       </c>
       <c r="I15" s="13" t="n">
         <f aca="false">Dynamics!J31</f>
-        <v>112.811366374384</v>
+        <v>92.1592512411451</v>
       </c>
       <c r="J15" s="13" t="n">
         <f aca="false">Dynamics!K31</f>
-        <v>129.197526605728</v>
+        <v>113.861115763633</v>
       </c>
       <c r="K15" s="13" t="n">
         <f aca="false">Dynamics!L31</f>
-        <v>145.967943936108</v>
+        <v>138.223598928754</v>
       </c>
       <c r="L15" s="13" t="n">
         <f aca="false">Dynamics!M31</f>
-        <v>162.585787656227</v>
+        <v>161.691775942088</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7351,31 +7351,31 @@
       </c>
       <c r="F16" s="13" t="n">
         <f aca="false">Dynamics!G42</f>
-        <v>38.8631625125858</v>
+        <v>38.0790429120858</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">Dynamics!H42</f>
-        <v>57.0483665802446</v>
+        <v>47.0207993247361</v>
       </c>
       <c r="H16" s="13" t="n">
         <f aca="false">Dynamics!I42</f>
-        <v>83.4395140442294</v>
+        <v>60.961054171011</v>
       </c>
       <c r="I16" s="13" t="n">
         <f aca="false">Dynamics!J42</f>
-        <v>118.801437617868</v>
+        <v>84.5663297633593</v>
       </c>
       <c r="J16" s="13" t="n">
         <f aca="false">Dynamics!K42</f>
-        <v>161.965735856375</v>
+        <v>136.182165523763</v>
       </c>
       <c r="K16" s="13" t="n">
         <f aca="false">Dynamics!L42</f>
-        <v>211.891147670215</v>
+        <v>204.986135272513</v>
       </c>
       <c r="L16" s="13" t="n">
         <f aca="false">Dynamics!M42</f>
-        <v>265.970138325472</v>
+        <v>283.244164629685</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7396,35 +7396,35 @@
       </c>
       <c r="E17" s="13" t="n">
         <f aca="false">Dynamics!F53</f>
-        <v>372.845896224325</v>
+        <v>367.20202040868</v>
       </c>
       <c r="F17" s="13" t="n">
         <f aca="false">Dynamics!G53</f>
-        <v>447.921231039373</v>
+        <v>373.715099393545</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">Dynamics!H53</f>
-        <v>535.418990376916</v>
+        <v>382.779441600897</v>
       </c>
       <c r="H17" s="13" t="n">
         <f aca="false">Dynamics!I53</f>
-        <v>595.96851740206</v>
+        <v>416.332652000454</v>
       </c>
       <c r="I17" s="13" t="n">
         <f aca="false">Dynamics!J53</f>
-        <v>640.460496505926</v>
+        <v>518.23627267686</v>
       </c>
       <c r="J17" s="13" t="n">
         <f aca="false">Dynamics!K53</f>
-        <v>683.92582902353</v>
+        <v>620.065334135792</v>
       </c>
       <c r="K17" s="13" t="n">
         <f aca="false">Dynamics!L53</f>
-        <v>730.076626053139</v>
+        <v>706.315473732858</v>
       </c>
       <c r="L17" s="13" t="n">
         <f aca="false">Dynamics!M53</f>
-        <v>774.505836010781</v>
+        <v>759.827524596415</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7453,27 +7453,27 @@
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">Dynamics!H64</f>
-        <v>70.4716911324647</v>
+        <v>69.4250795966256</v>
       </c>
       <c r="H18" s="13" t="n">
         <f aca="false">Dynamics!I64</f>
-        <v>86.4089066187107</v>
+        <v>76.2669147506252</v>
       </c>
       <c r="I18" s="13" t="n">
         <f aca="false">Dynamics!J64</f>
-        <v>111.55398314447</v>
+        <v>86.3475403019533</v>
       </c>
       <c r="J18" s="13" t="n">
         <f aca="false">Dynamics!K64</f>
-        <v>143.099314195527</v>
+        <v>106.609437013884</v>
       </c>
       <c r="K18" s="13" t="n">
         <f aca="false">Dynamics!L64</f>
-        <v>185.312976694668</v>
+        <v>151.027672634075</v>
       </c>
       <c r="L18" s="13" t="n">
         <f aca="false">Dynamics!M64</f>
-        <v>228.894685267663</v>
+        <v>206.50603617164</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7503,31 +7503,31 @@
       </c>
       <c r="F21" s="13" t="n">
         <f aca="false">Dynamics!G11</f>
-        <v>-1.24898048013472</v>
+        <v>-1.38901270864005</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">Dynamics!H11</f>
-        <v>0.640091749889621</v>
+        <v>-1.3546278918617</v>
       </c>
       <c r="H21" s="13" t="n">
         <f aca="false">Dynamics!I11</f>
-        <v>4.06226678766274</v>
+        <v>-0.212673566792859</v>
       </c>
       <c r="I21" s="13" t="n">
         <f aca="false">Dynamics!J11</f>
-        <v>13.5973828031006</v>
+        <v>6.80821201680257</v>
       </c>
       <c r="J21" s="13" t="n">
         <f aca="false">Dynamics!K11</f>
-        <v>26.5117810565617</v>
+        <v>20.2554323496811</v>
       </c>
       <c r="K21" s="13" t="n">
         <f aca="false">Dynamics!L11</f>
-        <v>42.2596881267166</v>
+        <v>37.4804104390084</v>
       </c>
       <c r="L21" s="13" t="n">
         <f aca="false">Dynamics!M11</f>
-        <v>59.64358455473</v>
+        <v>57.4070422942264</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7544,39 +7544,39 @@
       </c>
       <c r="D22" s="13" t="n">
         <f aca="false">Dynamics!E22</f>
-        <v>15.8531476766989</v>
+        <v>15.0723744473576</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">Dynamics!F22</f>
-        <v>30.8773086564933</v>
+        <v>19.1562215538352</v>
       </c>
       <c r="F22" s="13" t="n">
         <f aca="false">Dynamics!G22</f>
-        <v>61.5205786586931</v>
+        <v>34.6134631954567</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">Dynamics!H22</f>
-        <v>110.53391043471</v>
+        <v>67.5205996763273</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">Dynamics!I22</f>
-        <v>168.331274938205</v>
+        <v>135.133052010671</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">Dynamics!J22</f>
-        <v>235.058311133993</v>
+        <v>218.008811679595</v>
       </c>
       <c r="J22" s="13" t="n">
         <f aca="false">Dynamics!K22</f>
-        <v>294.406278237303</v>
+        <v>303.148838462092</v>
       </c>
       <c r="K22" s="13" t="n">
         <f aca="false">Dynamics!L22</f>
-        <v>347.874025602136</v>
+        <v>378.514716973411</v>
       </c>
       <c r="L22" s="13" t="n">
         <f aca="false">Dynamics!M22</f>
-        <v>392.360577261666</v>
+        <v>439.66394698948</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7597,35 +7597,35 @@
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">Dynamics!F33</f>
-        <v>-11.3801623422023</v>
+        <v>-11.453533526154</v>
       </c>
       <c r="F23" s="13" t="n">
         <f aca="false">Dynamics!G33</f>
-        <v>-10.9481524790998</v>
+        <v>-12.4789578192194</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">Dynamics!H33</f>
-        <v>-9.0082768655934</v>
+        <v>-12.6635243126684</v>
       </c>
       <c r="H23" s="13" t="n">
         <f aca="false">Dynamics!I33</f>
-        <v>-5.42892527297296</v>
+        <v>-11.2504095181181</v>
       </c>
       <c r="I23" s="13" t="n">
         <f aca="false">Dynamics!J33</f>
-        <v>2.44635228909446</v>
+        <v>-2.61464869872807</v>
       </c>
       <c r="J23" s="13" t="n">
         <f aca="false">Dynamics!K33</f>
-        <v>13.0332752142127</v>
+        <v>10.4568147054286</v>
       </c>
       <c r="K23" s="13" t="n">
         <f aca="false">Dynamics!L33</f>
-        <v>25.6871506252367</v>
+        <v>27.0154152389962</v>
       </c>
       <c r="L23" s="13" t="n">
         <f aca="false">Dynamics!M33</f>
-        <v>39.6889600345054</v>
+        <v>44.8299480370181</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7650,31 +7650,31 @@
       </c>
       <c r="F24" s="13" t="n">
         <f aca="false">Dynamics!G44</f>
-        <v>-26.005097448887</v>
+        <v>-26.226935252054</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">Dynamics!H44</f>
-        <v>-19.5059014463545</v>
+        <v>-23.556866405409</v>
       </c>
       <c r="H24" s="13" t="n">
         <f aca="false">Dynamics!I44</f>
-        <v>-6.32621867480042</v>
+        <v>-17.1211868352275</v>
       </c>
       <c r="I24" s="13" t="n">
         <f aca="false">Dynamics!J44</f>
-        <v>14.4344251780161</v>
+        <v>-3.78760526461738</v>
       </c>
       <c r="J24" s="13" t="n">
         <f aca="false">Dynamics!K44</f>
-        <v>45.225770761512</v>
+        <v>33.2338788323841</v>
       </c>
       <c r="K24" s="13" t="n">
         <f aca="false">Dynamics!L44</f>
-        <v>84.6268872950972</v>
+        <v>87.5632188532965</v>
       </c>
       <c r="L24" s="13" t="n">
         <f aca="false">Dynamics!M44</f>
-        <v>128.713545634631</v>
+        <v>151.716877146872</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7695,35 +7695,35 @@
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">Dynamics!F55</f>
-        <v>92.9922272787662</v>
+        <v>90.8428500007444</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">Dynamics!G55</f>
-        <v>118.072684549662</v>
+        <v>89.7625343360509</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">Dynamics!H55</f>
-        <v>148.516615338315</v>
+        <v>90.4168192098907</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">Dynamics!I55</f>
-        <v>168.988966964468</v>
+        <v>101.210910076185</v>
       </c>
       <c r="I25" s="13" t="n">
         <f aca="false">Dynamics!J55</f>
-        <v>183.379277888107</v>
+        <v>139.28374006689</v>
       </c>
       <c r="J25" s="13" t="n">
         <f aca="false">Dynamics!K55</f>
-        <v>197.230100832342</v>
+        <v>177.239738894763</v>
       </c>
       <c r="K25" s="13" t="n">
         <f aca="false">Dynamics!L55</f>
-        <v>211.750284877456</v>
+        <v>208.598640506586</v>
       </c>
       <c r="L25" s="13" t="n">
         <f aca="false">Dynamics!M55</f>
-        <v>225.030049879965</v>
+        <v>226.282442326827</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7752,27 +7752,27 @@
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">Dynamics!H66</f>
-        <v>-10.7989784626719</v>
+        <v>-11.188103385759</v>
       </c>
       <c r="H26" s="13" t="n">
         <f aca="false">Dynamics!I66</f>
-        <v>-3.20829530273441</v>
+        <v>-7.59557527685132</v>
       </c>
       <c r="I26" s="13" t="n">
         <f aca="false">Dynamics!J66</f>
-        <v>10.9443389373844</v>
+        <v>-1.16225719685809</v>
       </c>
       <c r="J26" s="13" t="n">
         <f aca="false">Dynamics!K66</f>
-        <v>32.3461422731247</v>
+        <v>13.5455148552129</v>
       </c>
       <c r="K26" s="13" t="n">
         <f aca="false">Dynamics!L66</f>
-        <v>63.646042838966</v>
+        <v>46.4271627839599</v>
       </c>
       <c r="L26" s="13" t="n">
         <f aca="false">Dynamics!M66</f>
-        <v>98.6576777088208</v>
+        <v>90.0052767464579</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7802,31 +7802,31 @@
       </c>
       <c r="F29" s="13" t="n">
         <f aca="false">Dynamics!G3</f>
-        <v>184.112133293435</v>
+        <v>183.737133293435</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">Dynamics!H3</f>
-        <v>178.026620362775</v>
+        <v>173.301745362775</v>
       </c>
       <c r="H29" s="13" t="n">
         <f aca="false">Dynamics!I3</f>
-        <v>172.973836798469</v>
+        <v>163.690528423469</v>
       </c>
       <c r="I29" s="13" t="n">
         <f aca="false">Dynamics!J3</f>
-        <v>169.509589732972</v>
+        <v>156.098263019097</v>
       </c>
       <c r="J29" s="13" t="n">
         <f aca="false">Dynamics!K3</f>
-        <v>165.652447220863</v>
+        <v>153.139679396817</v>
       </c>
       <c r="K29" s="13" t="n">
         <f aca="false">Dynamics!L3</f>
-        <v>161.428733257065</v>
+        <v>150.75432087723</v>
       </c>
       <c r="L29" s="13" t="n">
         <f aca="false">Dynamics!M3</f>
-        <v>156.238008128841</v>
+        <v>148.153781378456</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7843,39 +7843,39 @@
       </c>
       <c r="D30" s="13" t="n">
         <f aca="false">Dynamics!E14</f>
-        <v>135.38668</v>
+        <v>133.38668</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">Dynamics!F14</f>
-        <v>161.31577244</v>
+        <v>134.44977244</v>
       </c>
       <c r="F30" s="13" t="n">
         <f aca="false">Dynamics!G14</f>
-        <v>190.50761568652</v>
+        <v>136.44163768652</v>
       </c>
       <c r="G30" s="13" t="n">
         <f aca="false">Dynamics!H14</f>
-        <v>222.743605435523</v>
+        <v>145.300047961523</v>
       </c>
       <c r="H30" s="13" t="n">
         <f aca="false">Dynamics!I14</f>
-        <v>247.819783871343</v>
+        <v>175.564944748101</v>
       </c>
       <c r="I30" s="13" t="n">
         <f aca="false">Dynamics!J14</f>
-        <v>271.215858351963</v>
+        <v>206.802093449978</v>
       </c>
       <c r="J30" s="13" t="n">
         <f aca="false">Dynamics!K14</f>
-        <v>283.044395842382</v>
+        <v>232.94635318883</v>
       </c>
       <c r="K30" s="13" t="n">
         <f aca="false">Dynamics!L14</f>
-        <v>289.080421320942</v>
+        <v>250.338947525178</v>
       </c>
       <c r="L30" s="13" t="n">
         <f aca="false">Dynamics!M14</f>
-        <v>289.712033092439</v>
+        <v>259.566238040991</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7896,35 +7896,35 @@
       </c>
       <c r="E31" s="13" t="n">
         <f aca="false">Dynamics!F25</f>
-        <v>37.12584948</v>
+        <v>36.92584948</v>
       </c>
       <c r="F31" s="13" t="n">
         <f aca="false">Dynamics!G25</f>
-        <v>39.63841756484</v>
+        <v>36.05181756484</v>
       </c>
       <c r="G31" s="13" t="n">
         <f aca="false">Dynamics!H25</f>
-        <v>42.9826435879957</v>
+        <v>35.2363457879957</v>
       </c>
       <c r="H31" s="13" t="n">
         <f aca="false">Dynamics!I25</f>
-        <v>47.1028064676</v>
+        <v>35.6755106202</v>
       </c>
       <c r="I31" s="13" t="n">
         <f aca="false">Dynamics!J25</f>
-        <v>50.9469184342708</v>
+        <v>39.8852514086466</v>
       </c>
       <c r="J31" s="13" t="n">
         <f aca="false">Dynamics!K25</f>
-        <v>53.5334748991747</v>
+        <v>44.2129395642673</v>
       </c>
       <c r="K31" s="13" t="n">
         <f aca="false">Dynamics!L25</f>
-        <v>54.94673208093</v>
+        <v>48.0506726134614</v>
       </c>
       <c r="L31" s="13" t="n">
         <f aca="false">Dynamics!M25</f>
-        <v>55.2653010315077</v>
+        <v>50.4312775483595</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7949,31 +7949,31 @@
       </c>
       <c r="F32" s="13" t="n">
         <f aca="false">Dynamics!G36</f>
-        <v>6.60837326139267</v>
+        <v>6.47503992805934</v>
       </c>
       <c r="G32" s="13" t="n">
         <f aca="false">Dynamics!H36</f>
-        <v>8.16561225287936</v>
+        <v>6.70787891954603</v>
       </c>
       <c r="H32" s="13" t="n">
         <f aca="false">Dynamics!I36</f>
-        <v>9.95184956526978</v>
+        <v>6.99178436526978</v>
       </c>
       <c r="I32" s="13" t="n">
         <f aca="false">Dynamics!J36</f>
-        <v>11.9517423110634</v>
+        <v>7.7233348127967</v>
       </c>
       <c r="J32" s="13" t="n">
         <f aca="false">Dynamics!K36</f>
-        <v>13.4843089095555</v>
+        <v>9.60587138033933</v>
       </c>
       <c r="K32" s="13" t="n">
         <f aca="false">Dynamics!L36</f>
-        <v>14.5808602126152</v>
+        <v>11.5622779978566</v>
       </c>
       <c r="L32" s="13" t="n">
         <f aca="false">Dynamics!M36</f>
-        <v>15.2706092450367</v>
+        <v>13.2542720386669</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7994,35 +7994,35 @@
       </c>
       <c r="E33" s="13" t="n">
         <f aca="false">Dynamics!F47</f>
-        <v>396.37218295</v>
+        <v>390.37218295</v>
       </c>
       <c r="F33" s="13" t="n">
         <f aca="false">Dynamics!G47</f>
-        <v>479.81524669235</v>
+        <v>400.21724669235</v>
       </c>
       <c r="G33" s="13" t="n">
         <f aca="false">Dynamics!H47</f>
-        <v>577.667625163963</v>
+        <v>411.402691163963</v>
       </c>
       <c r="H33" s="13" t="n">
         <f aca="false">Dynamics!I47</f>
-        <v>648</v>
+        <v>447.838710855977</v>
       </c>
       <c r="I33" s="13" t="n">
         <f aca="false">Dynamics!J47</f>
-        <v>702</v>
+        <v>557.833517228627</v>
       </c>
       <c r="J33" s="13" t="n">
         <f aca="false">Dynamics!K47</f>
-        <v>756</v>
+        <v>670.458671574309</v>
       </c>
       <c r="K33" s="13" t="n">
         <f aca="false">Dynamics!L47</f>
-        <v>814.5</v>
+        <v>769.53794057883</v>
       </c>
       <c r="L33" s="13" t="n">
         <f aca="false">Dynamics!M47</f>
-        <v>873</v>
+        <v>835.978898560049</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8051,27 +8051,27 @@
       </c>
       <c r="G34" s="13" t="n">
         <f aca="false">Dynamics!H58</f>
-        <v>11.2221979724254</v>
+        <v>11.0555313057587</v>
       </c>
       <c r="H34" s="13" t="n">
         <f aca="false">Dynamics!I58</f>
-        <v>12.5536440416062</v>
+        <v>11.0648107082729</v>
       </c>
       <c r="I34" s="13" t="n">
         <f aca="false">Dynamics!J58</f>
-        <v>14.6292165574853</v>
+        <v>11.1568017241519</v>
       </c>
       <c r="J34" s="13" t="n">
         <f aca="false">Dynamics!K58</f>
-        <v>16.5657257148004</v>
+        <v>11.7426293419671</v>
       </c>
       <c r="K34" s="13" t="n">
         <f aca="false">Dynamics!L58</f>
-        <v>18.7891554252421</v>
+        <v>13.9558731760553</v>
       </c>
       <c r="L34" s="13" t="n">
         <f aca="false">Dynamics!M58</f>
-        <v>20.4469486784176</v>
+        <v>16.3541630065929</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8101,31 +8101,31 @@
       </c>
       <c r="F37" s="13" t="n">
         <f aca="false">Dynamics!G2</f>
-        <v>184.112133293435</v>
+        <v>183.737133293435</v>
       </c>
       <c r="G37" s="13" t="n">
         <f aca="false">Dynamics!H2</f>
-        <v>178.026620362775</v>
+        <v>173.301745362775</v>
       </c>
       <c r="H37" s="13" t="n">
         <f aca="false">Dynamics!I2</f>
-        <v>172.973836798469</v>
+        <v>163.690528423469</v>
       </c>
       <c r="I37" s="13" t="n">
         <f aca="false">Dynamics!J2</f>
-        <v>169.509589732972</v>
+        <v>156.098263019097</v>
       </c>
       <c r="J37" s="13" t="n">
         <f aca="false">Dynamics!K2</f>
-        <v>165.652447220863</v>
+        <v>153.139679396817</v>
       </c>
       <c r="K37" s="13" t="n">
         <f aca="false">Dynamics!L2</f>
-        <v>161.428733257065</v>
+        <v>150.75432087723</v>
       </c>
       <c r="L37" s="13" t="n">
         <f aca="false">Dynamics!M2</f>
-        <v>156.238008128841</v>
+        <v>148.153781378456</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8142,39 +8142,39 @@
       </c>
       <c r="D38" s="13" t="n">
         <f aca="false">Dynamics!E13</f>
-        <v>135.38668</v>
+        <v>133.38668</v>
       </c>
       <c r="E38" s="13" t="n">
         <f aca="false">Dynamics!F13</f>
-        <v>161.31577244</v>
+        <v>134.44977244</v>
       </c>
       <c r="F38" s="13" t="n">
         <f aca="false">Dynamics!G13</f>
-        <v>190.50761568652</v>
+        <v>136.44163768652</v>
       </c>
       <c r="G38" s="13" t="n">
         <f aca="false">Dynamics!H13</f>
-        <v>222.743605435523</v>
+        <v>145.300047961523</v>
       </c>
       <c r="H38" s="13" t="n">
         <f aca="false">Dynamics!I13</f>
-        <v>247.819783871343</v>
+        <v>175.564944748101</v>
       </c>
       <c r="I38" s="13" t="n">
         <f aca="false">Dynamics!J13</f>
-        <v>271.215858351963</v>
+        <v>206.802093449978</v>
       </c>
       <c r="J38" s="13" t="n">
         <f aca="false">Dynamics!K13</f>
-        <v>283.044395842382</v>
+        <v>232.94635318883</v>
       </c>
       <c r="K38" s="13" t="n">
         <f aca="false">Dynamics!L13</f>
-        <v>289.080421320942</v>
+        <v>250.338947525178</v>
       </c>
       <c r="L38" s="13" t="n">
         <f aca="false">Dynamics!M13</f>
-        <v>289.712033092439</v>
+        <v>259.566238040991</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8195,35 +8195,35 @@
       </c>
       <c r="E39" s="13" t="n">
         <f aca="false">Dynamics!F24</f>
-        <v>37.12584948</v>
+        <v>36.92584948</v>
       </c>
       <c r="F39" s="13" t="n">
         <f aca="false">Dynamics!G24</f>
-        <v>39.63841756484</v>
+        <v>36.05181756484</v>
       </c>
       <c r="G39" s="13" t="n">
         <f aca="false">Dynamics!H24</f>
-        <v>42.9826435879957</v>
+        <v>35.2363457879957</v>
       </c>
       <c r="H39" s="13" t="n">
         <f aca="false">Dynamics!I24</f>
-        <v>47.1028064676</v>
+        <v>35.6755106202</v>
       </c>
       <c r="I39" s="13" t="n">
         <f aca="false">Dynamics!J24</f>
-        <v>50.9469184342708</v>
+        <v>39.8852514086466</v>
       </c>
       <c r="J39" s="13" t="n">
         <f aca="false">Dynamics!K24</f>
-        <v>53.5334748991747</v>
+        <v>44.2129395642673</v>
       </c>
       <c r="K39" s="13" t="n">
         <f aca="false">Dynamics!L24</f>
-        <v>54.94673208093</v>
+        <v>48.0506726134614</v>
       </c>
       <c r="L39" s="13" t="n">
         <f aca="false">Dynamics!M24</f>
-        <v>55.2653010315077</v>
+        <v>50.4312775483595</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8248,31 +8248,31 @@
       </c>
       <c r="F40" s="13" t="n">
         <f aca="false">Dynamics!G35</f>
-        <v>6.60837326139267</v>
+        <v>6.47503992805934</v>
       </c>
       <c r="G40" s="13" t="n">
         <f aca="false">Dynamics!H35</f>
-        <v>8.16561225287936</v>
+        <v>6.70787891954603</v>
       </c>
       <c r="H40" s="13" t="n">
         <f aca="false">Dynamics!I35</f>
-        <v>9.95184956526978</v>
+        <v>6.99178436526978</v>
       </c>
       <c r="I40" s="13" t="n">
         <f aca="false">Dynamics!J35</f>
-        <v>11.9517423110634</v>
+        <v>7.7233348127967</v>
       </c>
       <c r="J40" s="13" t="n">
         <f aca="false">Dynamics!K35</f>
-        <v>13.4843089095555</v>
+        <v>9.60587138033933</v>
       </c>
       <c r="K40" s="13" t="n">
         <f aca="false">Dynamics!L35</f>
-        <v>14.5808602126152</v>
+        <v>11.5622779978566</v>
       </c>
       <c r="L40" s="13" t="n">
         <f aca="false">Dynamics!M35</f>
-        <v>15.2706092450367</v>
+        <v>13.2542720386669</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8293,35 +8293,35 @@
       </c>
       <c r="E41" s="13" t="n">
         <f aca="false">Dynamics!F46</f>
-        <v>396.37218295</v>
+        <v>390.37218295</v>
       </c>
       <c r="F41" s="13" t="n">
         <f aca="false">Dynamics!G46</f>
-        <v>479.81524669235</v>
+        <v>400.21724669235</v>
       </c>
       <c r="G41" s="13" t="n">
         <f aca="false">Dynamics!H46</f>
-        <v>577.667625163963</v>
+        <v>411.402691163963</v>
       </c>
       <c r="H41" s="13" t="n">
         <f aca="false">Dynamics!I46</f>
-        <v>688.963894277977</v>
+        <v>447.838710855977</v>
       </c>
       <c r="I41" s="13" t="n">
         <f aca="false">Dynamics!J46</f>
-        <v>782.803313361353</v>
+        <v>557.833517228627</v>
       </c>
       <c r="J41" s="13" t="n">
         <f aca="false">Dynamics!K46</f>
-        <v>850.355491366142</v>
+        <v>670.458671574309</v>
       </c>
       <c r="K41" s="13" t="n">
         <f aca="false">Dynamics!L46</f>
-        <v>903.381673444611</v>
+        <v>769.53794057883</v>
       </c>
       <c r="L41" s="13" t="n">
         <f aca="false">Dynamics!M46</f>
-        <v>932.855101323822</v>
+        <v>835.978898560049</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8350,27 +8350,27 @@
       </c>
       <c r="G42" s="13" t="n">
         <f aca="false">Dynamics!H57</f>
-        <v>11.2221979724254</v>
+        <v>11.0555313057587</v>
       </c>
       <c r="H42" s="13" t="n">
         <f aca="false">Dynamics!I57</f>
-        <v>12.5536440416062</v>
+        <v>11.0648107082729</v>
       </c>
       <c r="I42" s="13" t="n">
         <f aca="false">Dynamics!J57</f>
-        <v>14.6292165574853</v>
+        <v>11.1568017241519</v>
       </c>
       <c r="J42" s="13" t="n">
         <f aca="false">Dynamics!K57</f>
-        <v>16.5657257148004</v>
+        <v>11.7426293419671</v>
       </c>
       <c r="K42" s="13" t="n">
         <f aca="false">Dynamics!L57</f>
-        <v>18.7891554252421</v>
+        <v>13.9558731760553</v>
       </c>
       <c r="L42" s="13" t="n">
         <f aca="false">Dynamics!M57</f>
-        <v>20.4469486784176</v>
+        <v>16.3541630065929</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="B47" s="13" t="n">
         <f aca="false">Financials!B22</f>
-        <v>9265.16281994792</v>
+        <v>9823.00522849734</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="B48" s="20" t="n">
         <f aca="false">Financials!B25</f>
-        <v>252.715092162442</v>
+        <v>359.494820102299</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">Financials!B26</f>
-        <v>3994.75571709648</v>
+        <v>4326.83844247624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: PM scenario update — USS/SPN/ANS price, cost, yield (v1.2.5)
Pull updated scenario files and reference data from project folder:
  USS: basePrice 2.00→2.40, baseUnitCost 1.70→1.40
  SPN: basePrice 1.50→1.80, yield 0.85→0.92
  ANS: basePrice 1.00→1.15, baseUnitCost 0.60→0.45

Regenerate growth_baseline_fixture.csv to match new defaults.
All 68 calibration and unit tests pass (4 pre-existing skips unchanged).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/reference/sps_reference_model.xlsx
+++ b/reference/sps_reference_model.xlsx
@@ -1476,7 +1476,7 @@
         <v>0.45</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0.85</v>
+        <v>0.92</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>0.75</v>
@@ -1565,7 +1565,7 @@
         <v>74</v>
       </c>
       <c r="B25" s="7" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="C25" s="7" t="n">
         <v>1.1</v>
@@ -1577,7 +1577,7 @@
         <v>4.8</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>4.5</v>
@@ -1634,10 +1634,10 @@
         <v>77</v>
       </c>
       <c r="B28" s="7" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>2</v>
@@ -1646,7 +1646,7 @@
         <v>6</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>1</v>
+        <v>1.15</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>6</v>
@@ -3122,47 +3122,47 @@
       </c>
       <c r="C5" s="12" t="n">
         <f aca="false">Inputs!B25*(C4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="D5" s="12" t="n">
         <f aca="false">Inputs!B25*(D4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.66328889660176</v>
+        <v>1.36976732661322</v>
       </c>
       <c r="E5" s="12" t="n">
         <f aca="false">Inputs!B25*(E4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.63386220053255</v>
+        <v>1.34553357690916</v>
       </c>
       <c r="F5" s="12" t="n">
         <f aca="false">Inputs!B25*(F4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.60964515931722</v>
+        <v>1.32559013120242</v>
       </c>
       <c r="G5" s="12" t="n">
         <f aca="false">Inputs!B25*(G4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.5890031139677</v>
+        <v>1.30859079973811</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">Inputs!B25*(H4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.5711465430386</v>
+        <v>1.29388538838473</v>
       </c>
       <c r="I5" s="12" t="n">
         <f aca="false">Inputs!B25*(I4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.55524390924683</v>
+        <v>1.28078910173268</v>
       </c>
       <c r="J5" s="12" t="n">
         <f aca="false">Inputs!B25*(J4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.54090162734017</v>
+        <v>1.26897781075073</v>
       </c>
       <c r="K5" s="12" t="n">
         <f aca="false">Inputs!B25*(K4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.52777434758907</v>
+        <v>1.25816710977923</v>
       </c>
       <c r="L5" s="12" t="n">
         <f aca="false">Inputs!B25*(L4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.51573045069291</v>
+        <v>1.24824860645298</v>
       </c>
       <c r="M5" s="12" t="n">
         <f aca="false">Inputs!B25*(M4/Inputs!B27)^(-Inputs!B26)</f>
-        <v>1.50465970675635</v>
+        <v>1.23913152321111</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3171,47 +3171,47 @@
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">Inputs!B28</f>
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">C6*(1-Inputs!B29)+C8/MAX(C3,1)</f>
-        <v>1.98</v>
+        <v>2.376</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">D6*(1-Inputs!B29)+D8/MAX(D3,1)</f>
-        <v>1.9602</v>
+        <v>2.35224</v>
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">E6*(1-Inputs!B29)+E8/MAX(E3,1)</f>
-        <v>1.940598</v>
+        <v>2.3287176</v>
       </c>
       <c r="G6" s="12" t="n">
         <f aca="false">F6*(1-Inputs!B29)+F8/MAX(F3,1)</f>
-        <v>1.96243252071503</v>
+        <v>2.34667092471503</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">G6*(1-Inputs!B29)+G8/MAX(G3,1)</f>
-        <v>2.00255439367109</v>
+        <v>2.38295041363109</v>
       </c>
       <c r="I6" s="12" t="n">
         <f aca="false">H6*(1-Inputs!B29)+H8/MAX(H3,1)</f>
-        <v>2.0615058025707</v>
+        <v>2.4380978623311</v>
       </c>
       <c r="J6" s="12" t="n">
         <f aca="false">I6*(1-Inputs!B29)+I8/MAX(I3,1)</f>
-        <v>2.14076712076325</v>
+        <v>2.51359325992605</v>
       </c>
       <c r="K6" s="12" t="n">
         <f aca="false">J6*(1-Inputs!B29)+J8/MAX(J3,1)</f>
-        <v>2.22589029555936</v>
+        <v>2.59498817333052</v>
       </c>
       <c r="L6" s="12" t="n">
         <f aca="false">K6*(1-Inputs!B29)+K8/MAX(K3,1)</f>
-        <v>2.31243751229826</v>
+        <v>2.67784441129172</v>
       </c>
       <c r="M6" s="12" t="n">
         <f aca="false">L6*(1-Inputs!B29)+L8/MAX(L3,1)</f>
-        <v>2.40075550333293</v>
+        <v>2.76250833333646</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3315,47 +3315,47 @@
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">C6*C3</f>
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">D6*D3</f>
-        <v>434.1249</v>
+        <v>520.94988</v>
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">E6*E3</f>
-        <v>400.988146383</v>
+        <v>481.1857756596</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">F6*F3</f>
-        <v>376.445089919586</v>
+        <v>451.734107903503</v>
       </c>
       <c r="G9" s="10" t="n">
         <f aca="false">G6*G3</f>
-        <v>361.307637833258</v>
+        <v>432.050590086963</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">H6*H3</f>
-        <v>356.50799079789</v>
+        <v>424.228608630819</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">I6*I3</f>
-        <v>356.586568252961</v>
+        <v>421.727141737555</v>
       </c>
       <c r="J9" s="10" t="n">
         <f aca="false">J6*J3</f>
-        <v>362.880556354413</v>
+        <v>426.078162245627</v>
       </c>
       <c r="K9" s="10" t="n">
         <f aca="false">K6*K3</f>
-        <v>368.724174704576</v>
+        <v>429.866141421397</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">L6*L3</f>
-        <v>373.293858346427</v>
+        <v>432.281031174332</v>
       </c>
       <c r="M9" s="10" t="n">
         <f aca="false">M6*M3</f>
-        <v>375.089257845092</v>
+        <v>431.608799439813</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3364,47 +3364,47 @@
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">C5*C3</f>
-        <v>399.5</v>
+        <v>329</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">D5*D3</f>
-        <v>364.68440702442</v>
+        <v>300.328335196581</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">E5*E3</f>
-        <v>334.230882173654</v>
+        <v>275.248961790068</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">F5*F3</f>
-        <v>312.24551233063</v>
+        <v>257.143363095813</v>
       </c>
       <c r="G10" s="10" t="n">
         <f aca="false">G5*G3</f>
-        <v>292.554753122505</v>
+        <v>240.927443747945</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">H5*H3</f>
-        <v>279.70590915182</v>
+        <v>230.34604283091</v>
       </c>
       <c r="I10" s="10" t="n">
         <f aca="false">I5*I3</f>
-        <v>269.016506139873</v>
+        <v>221.543005056366</v>
       </c>
       <c r="J10" s="10" t="n">
         <f aca="false">J5*J3</f>
-        <v>261.1976026693</v>
+        <v>215.1039080806</v>
       </c>
       <c r="K10" s="10" t="n">
         <f aca="false">K5*K3</f>
-        <v>253.079559479386</v>
+        <v>208.41846074773</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">L5*L3</f>
-        <v>244.682446614516</v>
+        <v>201.503191329601</v>
       </c>
       <c r="M10" s="10" t="n">
         <f aca="false">M5*M3</f>
-        <v>235.085035495339</v>
+        <v>193.599440996161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3413,47 +3413,47 @@
       </c>
       <c r="C11" s="10" t="n">
         <f aca="false">C9-C10-Inputs!B39-Decisions!C19</f>
-        <v>20.5</v>
+        <v>185</v>
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">D9-D10-Inputs!C39-Decisions!D19</f>
-        <v>16.3404929755802</v>
+        <v>167.521544803419</v>
       </c>
       <c r="E11" s="10" t="n">
         <f aca="false">E9-E10-Inputs!D39-Decisions!E19</f>
-        <v>9.39726420934655</v>
+        <v>148.576813869532</v>
       </c>
       <c r="F11" s="10" t="n">
         <f aca="false">F9-F10-Inputs!E39-Decisions!F19</f>
-        <v>4.22957758895538</v>
+        <v>134.62074480769</v>
       </c>
       <c r="G11" s="10" t="n">
         <f aca="false">G9-G10-Inputs!F39-Decisions!G19</f>
-        <v>5.14288471075322</v>
+        <v>127.513146339018</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">H9-H10-Inputs!G39-Decisions!H19</f>
-        <v>7.17208164607029</v>
+        <v>124.252565799909</v>
       </c>
       <c r="I11" s="10" t="n">
         <f aca="false">I9-I10-Inputs!H39-Decisions!I19</f>
-        <v>13.080062113087</v>
+        <v>125.694136681189</v>
       </c>
       <c r="J11" s="10" t="n">
         <f aca="false">J9-J10-Inputs!I39-Decisions!J19</f>
-        <v>22.3829536851132</v>
+        <v>131.674254165026</v>
       </c>
       <c r="K11" s="10" t="n">
         <f aca="false">K9-K10-Inputs!J39-Decisions!K19</f>
-        <v>30.74461522519</v>
+        <v>136.547680673667</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">L9-L10-Inputs!K39-Decisions!L19</f>
-        <v>37.7814117319108</v>
+        <v>139.947839844731</v>
       </c>
       <c r="M11" s="10" t="n">
         <f aca="false">M9-M10-Inputs!L39-Decisions!M19</f>
-        <v>43.0042223497528</v>
+        <v>141.009358443652</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3661,47 +3661,47 @@
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">Inputs!C28</f>
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">C17*(1-Inputs!C29)+C19/MAX(C14,1)</f>
-        <v>1.4775</v>
+        <v>1.773</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">D17*(1-Inputs!C29)+D19/MAX(D14,1)</f>
-        <v>1.4553375</v>
+        <v>1.746405</v>
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">E17*(1-Inputs!C29)+E19/MAX(E14,1)</f>
-        <v>1.48890431997027</v>
+        <v>1.77560580747027</v>
       </c>
       <c r="G17" s="12" t="n">
         <f aca="false">F17*(1-Inputs!C29)+F19/MAX(F14,1)</f>
-        <v>1.52236195192643</v>
+        <v>1.80476291711393</v>
       </c>
       <c r="H17" s="12" t="n">
         <f aca="false">G17*(1-Inputs!C29)+G19/MAX(G14,1)</f>
-        <v>1.56767850307395</v>
+        <v>1.84584345378364</v>
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">H17*(1-Inputs!C29)+H19/MAX(H14,1)</f>
-        <v>1.59843081591685</v>
+        <v>1.87242329236589</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">I17*(1-Inputs!C29)+I19/MAX(I14,1)</f>
-        <v>1.61933102669467</v>
+        <v>1.88921361599697</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">J17*(1-Inputs!C29)+J19/MAX(J14,1)</f>
-        <v>1.63179028906297</v>
+        <v>1.89762463952574</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">K17*(1-Inputs!C29)+K19/MAX(K14,1)</f>
-        <v>1.63982858893379</v>
+        <v>1.90167542413962</v>
       </c>
       <c r="M17" s="12" t="n">
         <f aca="false">L17*(1-Inputs!C29)+L19/MAX(L14,1)</f>
-        <v>1.64594396037004</v>
+        <v>1.90386309304778</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,47 +3806,47 @@
       </c>
       <c r="C20" s="10" t="n">
         <f aca="false">C17*C14</f>
-        <v>180</v>
+        <v>216</v>
       </c>
       <c r="D20" s="10" t="n">
         <f aca="false">D17*D14</f>
-        <v>189.0609</v>
+        <v>226.87308</v>
       </c>
       <c r="E20" s="10" t="n">
         <f aca="false">E17*E14</f>
-        <v>197.0333124045</v>
+        <v>236.4399748854</v>
       </c>
       <c r="F20" s="10" t="n">
         <f aca="false">F17*F14</f>
-        <v>240.183750465257</v>
+        <v>286.433222381017</v>
       </c>
       <c r="G20" s="10" t="n">
         <f aca="false">G17*G14</f>
-        <v>235.216515404029</v>
+        <v>278.849615202722</v>
       </c>
       <c r="H20" s="10" t="n">
         <f aca="false">H17*H14</f>
-        <v>296.535176377208</v>
+        <v>349.151636039641</v>
       </c>
       <c r="I20" s="10" t="n">
         <f aca="false">I17*I14</f>
-        <v>346.03178740321</v>
+        <v>405.346275973246</v>
       </c>
       <c r="J20" s="10" t="n">
         <f aca="false">J17*J14</f>
-        <v>391.842278850273</v>
+        <v>457.147893990672</v>
       </c>
       <c r="K20" s="10" t="n">
         <f aca="false">K17*K14</f>
-        <v>417.355424646685</v>
+        <v>485.34664200267</v>
       </c>
       <c r="L20" s="10" t="n">
         <f aca="false">L17*L14</f>
-        <v>433.946326589705</v>
+        <v>503.238613011294</v>
       </c>
       <c r="M20" s="10" t="n">
         <f aca="false">M17*M14</f>
-        <v>442.592568495713</v>
+        <v>511.946747097495</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3904,47 +3904,47 @@
       </c>
       <c r="C22" s="10" t="n">
         <f aca="false">C20-C21-Inputs!B40-Decisions!C20</f>
-        <v>26.5</v>
+        <v>62.5</v>
       </c>
       <c r="D22" s="10" t="n">
         <f aca="false">D20-D21-Inputs!C40-Decisions!D20</f>
-        <v>27.1158940499523</v>
+        <v>64.9280740499523</v>
       </c>
       <c r="E22" s="10" t="n">
         <f aca="false">E20-E21-Inputs!D40-Decisions!E20</f>
-        <v>26.2456243040768</v>
+        <v>65.6522867849768</v>
       </c>
       <c r="F22" s="10" t="n">
         <f aca="false">F20-F21-Inputs!E40-Decisions!F20</f>
-        <v>41.1798841366883</v>
+        <v>87.4293560524479</v>
       </c>
       <c r="G22" s="10" t="n">
         <f aca="false">G20-G21-Inputs!F40-Decisions!G20</f>
-        <v>41.7157579339878</v>
+        <v>85.3488577326803</v>
       </c>
       <c r="H22" s="10" t="n">
         <f aca="false">H20-H21-Inputs!G40-Decisions!H20</f>
-        <v>65.5792667770498</v>
+        <v>118.195726439483</v>
       </c>
       <c r="I22" s="10" t="n">
         <f aca="false">I20-I21-Inputs!H40-Decisions!I20</f>
-        <v>86.0755154745097</v>
+        <v>145.390004044546</v>
       </c>
       <c r="J22" s="10" t="n">
         <f aca="false">J20-J21-Inputs!I40-Decisions!J20</f>
-        <v>105.402737312138</v>
+        <v>170.708352452536</v>
       </c>
       <c r="K22" s="10" t="n">
         <f aca="false">K20-K21-Inputs!J40-Decisions!K20</f>
-        <v>116.501440509386</v>
+        <v>184.492657865371</v>
       </c>
       <c r="L22" s="10" t="n">
         <f aca="false">L20-L21-Inputs!K40-Decisions!L20</f>
-        <v>123.340527806587</v>
+        <v>192.632814228175</v>
       </c>
       <c r="M22" s="10" t="n">
         <f aca="false">M20-M21-Inputs!L40-Decisions!M20</f>
-        <v>126.400638775888</v>
+        <v>195.75481737767</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5082,47 +5082,47 @@
       </c>
       <c r="C49" s="12" t="n">
         <f aca="false">Inputs!F25*(C48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="D49" s="12" t="n">
         <f aca="false">Inputs!F25*(D48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.597261992806544</v>
+        <v>0.447946494604908</v>
       </c>
       <c r="E49" s="12" t="n">
         <f aca="false">Inputs!F25*(E48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.594604899473062</v>
+        <v>0.445953674604796</v>
       </c>
       <c r="F49" s="12" t="n">
         <f aca="false">Inputs!F25*(F48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.59194805745454</v>
+        <v>0.443961043090905</v>
       </c>
       <c r="G49" s="12" t="n">
         <f aca="false">Inputs!F25*(G48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.589268440385567</v>
+        <v>0.441951330289175</v>
       </c>
       <c r="H49" s="12" t="n">
         <f aca="false">Inputs!F25*(H48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.586567550354507</v>
+        <v>0.43992566276588</v>
       </c>
       <c r="I49" s="12" t="n">
         <f aca="false">Inputs!F25*(I48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.583746126027667</v>
+        <v>0.43780959452075</v>
       </c>
       <c r="J49" s="12" t="n">
         <f aca="false">Inputs!F25*(J48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.580729213893658</v>
+        <v>0.435546910420243</v>
       </c>
       <c r="K49" s="12" t="n">
         <f aca="false">Inputs!F25*(K48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.57746033069914</v>
+        <v>0.433095248024355</v>
       </c>
       <c r="L49" s="12" t="n">
         <f aca="false">Inputs!F25*(L48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.573965968864345</v>
+        <v>0.430474476648259</v>
       </c>
       <c r="M49" s="12" t="n">
         <f aca="false">Inputs!F25*(M48/Inputs!F27)^(-Inputs!F26)</f>
-        <v>0.57009163173332</v>
+        <v>0.42756872379999</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5131,47 +5131,47 @@
       </c>
       <c r="C50" s="12" t="n">
         <f aca="false">Inputs!F28</f>
-        <v>1</v>
+        <v>1.15</v>
       </c>
       <c r="D50" s="12" t="n">
         <f aca="false">C50*(1-Inputs!F29)+C52/MAX(C47,1)</f>
-        <v>0.975</v>
+        <v>1.12125</v>
       </c>
       <c r="E50" s="12" t="n">
         <f aca="false">D50*(1-Inputs!F29)+D52/MAX(D47,1)</f>
-        <v>0.950625</v>
+        <v>1.09321875</v>
       </c>
       <c r="F50" s="12" t="n">
         <f aca="false">E50*(1-Inputs!F29)+E52/MAX(E47,1)</f>
-        <v>0.960106266415653</v>
+        <v>1.09913517266565</v>
       </c>
       <c r="G50" s="12" t="n">
         <f aca="false">F50*(1-Inputs!F29)+F52/MAX(F47,1)</f>
-        <v>0.967473206342249</v>
+        <v>1.103026389936</v>
       </c>
       <c r="H50" s="12" t="n">
         <f aca="false">G50*(1-Inputs!F29)+G52/MAX(G47,1)</f>
-        <v>0.976495397671883</v>
+        <v>1.10865975167579</v>
       </c>
       <c r="I50" s="12" t="n">
         <f aca="false">H50*(1-Inputs!F29)+H52/MAX(H47,1)</f>
-        <v>0.979013332880745</v>
+        <v>1.10787357803455</v>
       </c>
       <c r="J50" s="12" t="n">
         <f aca="false">I50*(1-Inputs!F29)+I52/MAX(I47,1)</f>
-        <v>0.97566006461564</v>
+        <v>1.1012988036406</v>
       </c>
       <c r="K50" s="12" t="n">
         <f aca="false">J50*(1-Inputs!F29)+J52/MAX(J47,1)</f>
-        <v>0.966808795741376</v>
+        <v>1.08930656629072</v>
       </c>
       <c r="L50" s="12" t="n">
         <f aca="false">K50*(1-Inputs!F29)+K52/MAX(K47,1)</f>
-        <v>0.954121086472228</v>
+        <v>1.07355641275783</v>
       </c>
       <c r="M50" s="12" t="n">
         <f aca="false">L50*(1-Inputs!F29)+L52/MAX(L47,1)</f>
-        <v>0.939280574572938</v>
+        <v>1.0557300177014</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5276,47 +5276,47 @@
       </c>
       <c r="C53" s="10" t="n">
         <f aca="false">C50*C47</f>
-        <v>140.4</v>
+        <v>161.46</v>
       </c>
       <c r="D53" s="10" t="n">
         <f aca="false">D50*D47</f>
-        <v>139.61025</v>
+        <v>160.5517875</v>
       </c>
       <c r="E53" s="10" t="n">
         <f aca="false">E50*E47</f>
-        <v>142.96449375</v>
+        <v>164.4091678125</v>
       </c>
       <c r="F53" s="10" t="n">
         <f aca="false">F50*F47</f>
-        <v>153.031337803991</v>
+        <v>175.191155171178</v>
       </c>
       <c r="G53" s="10" t="n">
         <f aca="false">G50*G47</f>
-        <v>163.435248747396</v>
+        <v>186.334248051888</v>
       </c>
       <c r="H53" s="10" t="n">
         <f aca="false">H50*H47</f>
-        <v>181.48166965732</v>
+        <v>206.044414848945</v>
       </c>
       <c r="I53" s="10" t="n">
         <f aca="false">I50*I47</f>
-        <v>205.56342950497</v>
+        <v>232.620215179915</v>
       </c>
       <c r="J53" s="10" t="n">
         <f aca="false">J50*J47</f>
-        <v>235.592635802739</v>
+        <v>265.930622115096</v>
       </c>
       <c r="K53" s="10" t="n">
         <f aca="false">K50*K47</f>
-        <v>266.172129555558</v>
+        <v>299.896990765497</v>
       </c>
       <c r="L53" s="10" t="n">
         <f aca="false">L50*L47</f>
-        <v>312.570067928302</v>
+        <v>351.697080819466</v>
       </c>
       <c r="M53" s="10" t="n">
         <f aca="false">M50*M47</f>
-        <v>369.249979476113</v>
+        <v>415.028584558776</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5325,47 +5325,47 @@
       </c>
       <c r="C54" s="10" t="n">
         <f aca="false">C49*C47</f>
-        <v>84.24</v>
+        <v>63.18</v>
       </c>
       <c r="D54" s="10" t="n">
         <f aca="false">D49*D47</f>
-        <v>85.521944749969</v>
+        <v>64.1414585624768</v>
       </c>
       <c r="E54" s="10" t="n">
         <f aca="false">E49*E47</f>
-        <v>89.4226308317538</v>
+        <v>67.0669731238153</v>
       </c>
       <c r="F54" s="10" t="n">
         <f aca="false">F49*F47</f>
-        <v>94.3506008776791</v>
+        <v>70.7629506582593</v>
       </c>
       <c r="G54" s="10" t="n">
         <f aca="false">G49*G47</f>
-        <v>99.5451176343338</v>
+        <v>74.6588382257503</v>
       </c>
       <c r="H54" s="10" t="n">
         <f aca="false">H49*H47</f>
-        <v>109.013579233385</v>
+        <v>81.7601844250388</v>
       </c>
       <c r="I54" s="10" t="n">
         <f aca="false">I49*I47</f>
-        <v>122.569174082029</v>
+        <v>91.9268805615219</v>
       </c>
       <c r="J54" s="10" t="n">
         <f aca="false">J49*J47</f>
-        <v>140.228683278902</v>
+        <v>105.171512459176</v>
       </c>
       <c r="K54" s="10" t="n">
         <f aca="false">K49*K47</f>
-        <v>158.98060364478</v>
+        <v>119.235452733585</v>
       </c>
       <c r="L54" s="10" t="n">
         <f aca="false">L49*L47</f>
-        <v>188.031251399959</v>
+        <v>141.02343854997</v>
       </c>
       <c r="M54" s="10" t="n">
         <f aca="false">M49*M47</f>
-        <v>224.114422267003</v>
+        <v>168.085816700252</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5374,47 +5374,47 @@
       </c>
       <c r="C55" s="10" t="n">
         <f aca="false">C53-C54-Inputs!B43-Decisions!C23</f>
-        <v>21.16</v>
+        <v>63.28</v>
       </c>
       <c r="D55" s="10" t="n">
         <f aca="false">D53-D54-Inputs!C43-Decisions!D23</f>
-        <v>14.868305250031</v>
+        <v>57.1903289375232</v>
       </c>
       <c r="E55" s="10" t="n">
         <f aca="false">E53-E54-Inputs!D43-Decisions!E23</f>
-        <v>11.2518629182462</v>
+        <v>55.0521946886847</v>
       </c>
       <c r="F55" s="10" t="n">
         <f aca="false">F53-F54-Inputs!E43-Decisions!F23</f>
-        <v>13.3207369263118</v>
+        <v>59.0682045129191</v>
       </c>
       <c r="G55" s="10" t="n">
         <f aca="false">G53-G54-Inputs!F43-Decisions!G23</f>
-        <v>14.4501311130624</v>
+        <v>62.235409826138</v>
       </c>
       <c r="H55" s="10" t="n">
         <f aca="false">H53-H54-Inputs!G43-Decisions!H23</f>
-        <v>19.1480904239344</v>
+        <v>70.9642304239066</v>
       </c>
       <c r="I55" s="10" t="n">
         <f aca="false">I53-I54-Inputs!H43-Decisions!I23</f>
-        <v>25.1942554229409</v>
+        <v>82.8933346183934</v>
       </c>
       <c r="J55" s="10" t="n">
         <f aca="false">J53-J54-Inputs!I43-Decisions!J23</f>
-        <v>33.643952523837</v>
+        <v>99.0391096559203</v>
       </c>
       <c r="K55" s="10" t="n">
         <f aca="false">K53-K54-Inputs!J43-Decisions!K23</f>
-        <v>41.2315259107779</v>
+        <v>114.701538031912</v>
       </c>
       <c r="L55" s="10" t="n">
         <f aca="false">L53-L54-Inputs!K43-Decisions!L23</f>
-        <v>54.2088165283426</v>
+        <v>140.343642269497</v>
       </c>
       <c r="M55" s="10" t="n">
         <f aca="false">M53-M54-Inputs!L43-Decisions!M23</f>
-        <v>70.3355572091107</v>
+        <v>172.142767858524</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5973,47 +5973,47 @@
       </c>
       <c r="B2" s="13" t="n">
         <f aca="false">Dynamics!C11</f>
-        <v>20.5</v>
+        <v>185</v>
       </c>
       <c r="C2" s="13" t="n">
         <f aca="false">Dynamics!D11</f>
-        <v>16.3404929755802</v>
+        <v>167.521544803419</v>
       </c>
       <c r="D2" s="13" t="n">
         <f aca="false">Dynamics!E11</f>
-        <v>9.39726420934655</v>
+        <v>148.576813869532</v>
       </c>
       <c r="E2" s="13" t="n">
         <f aca="false">Dynamics!F11</f>
-        <v>4.22957758895538</v>
+        <v>134.62074480769</v>
       </c>
       <c r="F2" s="13" t="n">
         <f aca="false">Dynamics!G11</f>
-        <v>5.14288471075322</v>
+        <v>127.513146339018</v>
       </c>
       <c r="G2" s="13" t="n">
         <f aca="false">Dynamics!H11</f>
-        <v>7.17208164607029</v>
+        <v>124.252565799909</v>
       </c>
       <c r="H2" s="13" t="n">
         <f aca="false">Dynamics!I11</f>
-        <v>13.080062113087</v>
+        <v>125.694136681189</v>
       </c>
       <c r="I2" s="13" t="n">
         <f aca="false">Dynamics!J11</f>
-        <v>22.3829536851132</v>
+        <v>131.674254165026</v>
       </c>
       <c r="J2" s="13" t="n">
         <f aca="false">Dynamics!K11</f>
-        <v>30.74461522519</v>
+        <v>136.547680673667</v>
       </c>
       <c r="K2" s="13" t="n">
         <f aca="false">Dynamics!L11</f>
-        <v>37.7814117319108</v>
+        <v>139.947839844731</v>
       </c>
       <c r="L2" s="13" t="n">
         <f aca="false">Dynamics!M11</f>
-        <v>43.0042223497528</v>
+        <v>141.009358443652</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6022,47 +6022,47 @@
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">Dynamics!C22</f>
-        <v>26.5</v>
+        <v>62.5</v>
       </c>
       <c r="C3" s="13" t="n">
         <f aca="false">Dynamics!D22</f>
-        <v>27.1158940499523</v>
+        <v>64.9280740499523</v>
       </c>
       <c r="D3" s="13" t="n">
         <f aca="false">Dynamics!E22</f>
-        <v>26.2456243040768</v>
+        <v>65.6522867849768</v>
       </c>
       <c r="E3" s="13" t="n">
         <f aca="false">Dynamics!F22</f>
-        <v>41.1798841366883</v>
+        <v>87.4293560524479</v>
       </c>
       <c r="F3" s="13" t="n">
         <f aca="false">Dynamics!G22</f>
-        <v>41.7157579339878</v>
+        <v>85.3488577326803</v>
       </c>
       <c r="G3" s="13" t="n">
         <f aca="false">Dynamics!H22</f>
-        <v>65.5792667770498</v>
+        <v>118.195726439483</v>
       </c>
       <c r="H3" s="13" t="n">
         <f aca="false">Dynamics!I22</f>
-        <v>86.0755154745097</v>
+        <v>145.390004044546</v>
       </c>
       <c r="I3" s="13" t="n">
         <f aca="false">Dynamics!J22</f>
-        <v>105.402737312138</v>
+        <v>170.708352452536</v>
       </c>
       <c r="J3" s="13" t="n">
         <f aca="false">Dynamics!K22</f>
-        <v>116.501440509386</v>
+        <v>184.492657865371</v>
       </c>
       <c r="K3" s="13" t="n">
         <f aca="false">Dynamics!L22</f>
-        <v>123.340527806587</v>
+        <v>192.632814228175</v>
       </c>
       <c r="L3" s="13" t="n">
         <f aca="false">Dynamics!M22</f>
-        <v>126.400638775888</v>
+        <v>195.75481737767</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6169,47 +6169,47 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">Dynamics!C55</f>
-        <v>21.16</v>
+        <v>63.28</v>
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">Dynamics!D55</f>
-        <v>14.868305250031</v>
+        <v>57.1903289375232</v>
       </c>
       <c r="D6" s="13" t="n">
         <f aca="false">Dynamics!E55</f>
-        <v>11.2518629182462</v>
+        <v>55.0521946886847</v>
       </c>
       <c r="E6" s="13" t="n">
         <f aca="false">Dynamics!F55</f>
-        <v>13.3207369263118</v>
+        <v>59.0682045129191</v>
       </c>
       <c r="F6" s="13" t="n">
         <f aca="false">Dynamics!G55</f>
-        <v>14.4501311130624</v>
+        <v>62.235409826138</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">Dynamics!H55</f>
-        <v>19.1480904239344</v>
+        <v>70.9642304239066</v>
       </c>
       <c r="H6" s="13" t="n">
         <f aca="false">Dynamics!I55</f>
-        <v>25.1942554229409</v>
+        <v>82.8933346183934</v>
       </c>
       <c r="I6" s="13" t="n">
         <f aca="false">Dynamics!J55</f>
-        <v>33.643952523837</v>
+        <v>99.0391096559203</v>
       </c>
       <c r="J6" s="13" t="n">
         <f aca="false">Dynamics!K55</f>
-        <v>41.2315259107779</v>
+        <v>114.701538031912</v>
       </c>
       <c r="K6" s="13" t="n">
         <f aca="false">Dynamics!L55</f>
-        <v>54.2088165283426</v>
+        <v>140.343642269497</v>
       </c>
       <c r="L6" s="13" t="n">
         <f aca="false">Dynamics!M55</f>
-        <v>70.3355572091107</v>
+        <v>172.142767858524</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6267,47 +6267,47 @@
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">SUM(B2:B7)</f>
-        <v>83.06</v>
+        <v>325.68</v>
       </c>
       <c r="C8" s="14" t="n">
         <f aca="false">SUM(C2:C7)</f>
-        <v>67.7549188441863</v>
+        <v>299.070174359517</v>
       </c>
       <c r="D8" s="14" t="n">
         <f aca="false">SUM(D2:D7)</f>
-        <v>48.6103626406531</v>
+        <v>270.996906552177</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">SUM(E2:E7)</f>
-        <v>49.0446150299653</v>
+        <v>271.432721751066</v>
       </c>
       <c r="F8" s="14" t="n">
         <f aca="false">SUM(F2:F7)</f>
-        <v>46.7335373711977</v>
+        <v>260.52217751123</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">SUM(G2:G7)</f>
-        <v>88.0300562823123</v>
+        <v>309.543140098557</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">SUM(H2:H7)</f>
-        <v>135.455796858559</v>
+        <v>365.08343919215</v>
       </c>
       <c r="I8" s="14" t="n">
         <f aca="false">SUM(I2:I7)</f>
-        <v>192.359021497629</v>
+        <v>432.351094250024</v>
       </c>
       <c r="J8" s="14" t="n">
         <f aca="false">SUM(J2:J7)</f>
-        <v>240.323942632287</v>
+        <v>487.588237557882</v>
       </c>
       <c r="K8" s="14" t="n">
         <f aca="false">SUM(K2:K7)</f>
-        <v>288.221843005757</v>
+        <v>545.81538328132</v>
       </c>
       <c r="L8" s="14" t="n">
         <f aca="false">SUM(L2:L7)</f>
-        <v>327.391865897276</v>
+        <v>596.558391242371</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6316,47 +6316,47 @@
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">Dynamics!C9+Dynamics!C20+Dynamics!C31+Dynamics!C42+Dynamics!C53+Dynamics!C64</f>
-        <v>978.4</v>
+        <v>1129.46</v>
       </c>
       <c r="C9" s="14" t="n">
         <f aca="false">Dynamics!D9+Dynamics!D20+Dynamics!D31+Dynamics!D42+Dynamics!D53+Dynamics!D64</f>
-        <v>936.20343</v>
+        <v>1081.7821275</v>
       </c>
       <c r="D9" s="14" t="n">
         <f aca="false">Dynamics!E9+Dynamics!E20+Dynamics!E31+Dynamics!E42+Dynamics!E53+Dynamics!E64</f>
-        <v>905.5523175858</v>
+        <v>1046.6012834058</v>
       </c>
       <c r="E9" s="14" t="n">
         <f aca="false">Dynamics!F9+Dynamics!F20+Dynamics!F31+Dynamics!F42+Dynamics!F53+Dynamics!F64</f>
-        <v>932.254574310729</v>
+        <v>1075.95288157759</v>
       </c>
       <c r="F9" s="14" t="n">
         <f aca="false">Dynamics!G9+Dynamics!G20+Dynamics!G31+Dynamics!G42+Dynamics!G53+Dynamics!G64</f>
-        <v>936.95436898183</v>
+        <v>1074.22942033872</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">Dynamics!H9+Dynamics!H20+Dynamics!H31+Dynamics!H42+Dynamics!H53+Dynamics!H64</f>
-        <v>1047.22088671583</v>
+        <v>1192.12070940282</v>
       </c>
       <c r="H9" s="14" t="n">
         <f aca="false">Dynamics!I9+Dynamics!I20+Dynamics!I31+Dynamics!I42+Dynamics!I53+Dynamics!I64</f>
-        <v>1166.76912820342</v>
+        <v>1318.280975933</v>
       </c>
       <c r="I9" s="14" t="n">
         <f aca="false">Dynamics!J9+Dynamics!J20+Dynamics!J31+Dynamics!J42+Dynamics!J53+Dynamics!J64</f>
-        <v>1304.18194659083</v>
+        <v>1463.02315393479</v>
       </c>
       <c r="J9" s="14" t="n">
         <f aca="false">Dynamics!K9+Dynamics!K20+Dynamics!K31+Dynamics!K42+Dynamics!K53+Dynamics!K64</f>
-        <v>1416.55118515123</v>
+        <v>1579.40923043398</v>
       </c>
       <c r="K9" s="14" t="n">
         <f aca="false">Dynamics!L9+Dynamics!L20+Dynamics!L31+Dynamics!L42+Dynamics!L53+Dynamics!L64</f>
-        <v>1532.55936936713</v>
+        <v>1699.96584150779</v>
       </c>
       <c r="L9" s="14" t="n">
         <f aca="false">Dynamics!M9+Dynamics!M20+Dynamics!M31+Dynamics!M42+Dynamics!M53+Dynamics!M64</f>
-        <v>1638.228350145</v>
+        <v>1809.88067542417</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6463,47 +6463,47 @@
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">B8*(1-Inputs!B3)+Inputs!B3*B11-B10</f>
-        <v>-34.246</v>
+        <v>184.112</v>
       </c>
       <c r="C12" s="14" t="n">
         <f aca="false">C8*(1-Inputs!B3)+Inputs!B3*C11-C10</f>
-        <v>-47.5205730402323</v>
+        <v>160.663156923566</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">D8*(1-Inputs!B3)+Inputs!B3*D11-D10</f>
-        <v>-169.250673623412</v>
+        <v>30.8972158969596</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">E8*(1-Inputs!B3)+Inputs!B3*E11-E10</f>
-        <v>-172.059846473031</v>
+        <v>28.0894495759597</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">F8*(1-Inputs!B3)+Inputs!B3*F11-F10</f>
-        <v>-244.139816365922</v>
+        <v>-51.7300402398928</v>
       </c>
       <c r="G12" s="14" t="n">
         <f aca="false">G8*(1-Inputs!B3)+Inputs!B3*G11-G10</f>
-        <v>-190.772949345919</v>
+        <v>8.58882608870101</v>
       </c>
       <c r="H12" s="14" t="n">
         <f aca="false">H8*(1-Inputs!B3)+Inputs!B3*H11-H10</f>
-        <v>-116.589782827297</v>
+        <v>90.0750952729349</v>
       </c>
       <c r="I12" s="14" t="n">
         <f aca="false">I8*(1-Inputs!B3)+Inputs!B3*I11-I10</f>
-        <v>-23.8768806521341</v>
+        <v>192.115984825021</v>
       </c>
       <c r="J12" s="14" t="n">
         <f aca="false">J8*(1-Inputs!B3)+Inputs!B3*J11-J10</f>
-        <v>52.2915483690579</v>
+        <v>274.829413802094</v>
       </c>
       <c r="K12" s="14" t="n">
         <f aca="false">K8*(1-Inputs!B3)+Inputs!B3*K11-K10</f>
-        <v>124.399658705181</v>
+        <v>356.233844953188</v>
       </c>
       <c r="L12" s="14" t="n">
         <f aca="false">L8*(1-Inputs!B3)+Inputs!B3*L11-L10</f>
-        <v>185.152679307549</v>
+        <v>427.402552118134</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6578,47 +6578,47 @@
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">B12*B17</f>
-        <v>-34.246</v>
+        <v>184.112</v>
       </c>
       <c r="C18" s="10" t="n">
         <f aca="false">C12*C17</f>
-        <v>-43.4453949901557</v>
+        <v>146.885314430029</v>
       </c>
       <c r="D18" s="10" t="n">
         <f aca="false">D12*D17</f>
-        <v>-141.466812363457</v>
+        <v>25.8251890540409</v>
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">E12*E17</f>
-        <v>-131.481840248741</v>
+        <v>21.4649297760491</v>
       </c>
       <c r="F18" s="10" t="n">
         <f aca="false">F12*F17</f>
-        <v>-170.563829178882</v>
+        <v>-36.1402489697512</v>
       </c>
       <c r="G18" s="10" t="n">
         <f aca="false">G12*G17</f>
-        <v>-121.850467213118</v>
+        <v>5.48585360402841</v>
       </c>
       <c r="H18" s="10" t="n">
         <f aca="false">H12*H17</f>
-        <v>-68.0821056374046</v>
+        <v>52.5989671046498</v>
       </c>
       <c r="I18" s="10" t="n">
         <f aca="false">I12*I17</f>
-        <v>-12.7471223809656</v>
+        <v>102.564736390111</v>
       </c>
       <c r="J18" s="10" t="n">
         <f aca="false">J12*J17</f>
-        <v>25.5227901272649</v>
+        <v>134.140480977241</v>
       </c>
       <c r="K18" s="10" t="n">
         <f aca="false">K12*K17</f>
-        <v>55.5108551213139</v>
+        <v>158.962215510334</v>
       </c>
       <c r="L18" s="10" t="n">
         <f aca="false">L12*L17</f>
-        <v>75.5354482233106</v>
+        <v>174.364440562075</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">L12*(1+Inputs!B9)</f>
-        <v>190.33695432816</v>
+        <v>439.369823577441</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="B22" s="14" t="n">
         <f aca="false">B21/($B$15-Inputs!B9)</f>
-        <v>2892.65888036717</v>
+        <v>6677.3529419064</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">B22*L17</f>
-        <v>1180.09788409671</v>
+        <v>2724.11314434367</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="B25" s="19" t="n">
         <f aca="false">SUM(C18:L18)</f>
-        <v>-533.068478540835</v>
+        <v>786.151878438808</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">B25+B23</f>
-        <v>647.029405555871</v>
+        <v>3510.26502278248</v>
       </c>
     </row>
   </sheetData>
@@ -6840,47 +6840,47 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">Financials!B9</f>
-        <v>978.4</v>
+        <v>1129.46</v>
       </c>
       <c r="C4" s="13" t="n">
         <f aca="false">Financials!C9</f>
-        <v>936.20343</v>
+        <v>1081.7821275</v>
       </c>
       <c r="D4" s="13" t="n">
         <f aca="false">Financials!D9</f>
-        <v>905.5523175858</v>
+        <v>1046.6012834058</v>
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">Financials!E9</f>
-        <v>932.254574310729</v>
+        <v>1075.95288157759</v>
       </c>
       <c r="F4" s="13" t="n">
         <f aca="false">Financials!F9</f>
-        <v>936.95436898183</v>
+        <v>1074.22942033872</v>
       </c>
       <c r="G4" s="13" t="n">
         <f aca="false">Financials!G9</f>
-        <v>1047.22088671583</v>
+        <v>1192.12070940282</v>
       </c>
       <c r="H4" s="13" t="n">
         <f aca="false">Financials!H9</f>
-        <v>1166.76912820342</v>
+        <v>1318.280975933</v>
       </c>
       <c r="I4" s="13" t="n">
         <f aca="false">Financials!I9</f>
-        <v>1304.18194659083</v>
+        <v>1463.02315393479</v>
       </c>
       <c r="J4" s="13" t="n">
         <f aca="false">Financials!J9</f>
-        <v>1416.55118515123</v>
+        <v>1579.40923043398</v>
       </c>
       <c r="K4" s="13" t="n">
         <f aca="false">Financials!K9</f>
-        <v>1532.55936936713</v>
+        <v>1699.96584150779</v>
       </c>
       <c r="L4" s="13" t="n">
         <f aca="false">Financials!L9</f>
-        <v>1638.228350145</v>
+        <v>1809.88067542417</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6889,47 +6889,47 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">Financials!B8</f>
-        <v>83.06</v>
+        <v>325.68</v>
       </c>
       <c r="C5" s="13" t="n">
         <f aca="false">Financials!C8</f>
-        <v>67.7549188441863</v>
+        <v>299.070174359517</v>
       </c>
       <c r="D5" s="13" t="n">
         <f aca="false">Financials!D8</f>
-        <v>48.6103626406531</v>
+        <v>270.996906552177</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">Financials!E8</f>
-        <v>49.0446150299653</v>
+        <v>271.432721751066</v>
       </c>
       <c r="F5" s="13" t="n">
         <f aca="false">Financials!F8</f>
-        <v>46.7335373711977</v>
+        <v>260.52217751123</v>
       </c>
       <c r="G5" s="13" t="n">
         <f aca="false">Financials!G8</f>
-        <v>88.0300562823123</v>
+        <v>309.543140098557</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">Financials!H8</f>
-        <v>135.455796858559</v>
+        <v>365.08343919215</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">Financials!I8</f>
-        <v>192.359021497629</v>
+        <v>432.351094250024</v>
       </c>
       <c r="J5" s="13" t="n">
         <f aca="false">Financials!J8</f>
-        <v>240.323942632287</v>
+        <v>487.588237557882</v>
       </c>
       <c r="K5" s="13" t="n">
         <f aca="false">Financials!K8</f>
-        <v>288.221843005757</v>
+        <v>545.81538328132</v>
       </c>
       <c r="L5" s="13" t="n">
         <f aca="false">Financials!L8</f>
-        <v>327.391865897276</v>
+        <v>596.558391242371</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7036,47 +7036,47 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">Financials!B12</f>
-        <v>-34.246</v>
+        <v>184.112</v>
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">Financials!C12</f>
-        <v>-47.5205730402323</v>
+        <v>160.663156923566</v>
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">Financials!D12</f>
-        <v>-169.250673623412</v>
+        <v>30.8972158969596</v>
       </c>
       <c r="E8" s="13" t="n">
         <f aca="false">Financials!E12</f>
-        <v>-172.059846473031</v>
+        <v>28.0894495759597</v>
       </c>
       <c r="F8" s="13" t="n">
         <f aca="false">Financials!F12</f>
-        <v>-244.139816365922</v>
+        <v>-51.7300402398928</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">Financials!G12</f>
-        <v>-190.772949345919</v>
+        <v>8.58882608870101</v>
       </c>
       <c r="H8" s="13" t="n">
         <f aca="false">Financials!H12</f>
-        <v>-116.589782827297</v>
+        <v>90.0750952729349</v>
       </c>
       <c r="I8" s="13" t="n">
         <f aca="false">Financials!I12</f>
-        <v>-23.8768806521341</v>
+        <v>192.115984825021</v>
       </c>
       <c r="J8" s="13" t="n">
         <f aca="false">Financials!J12</f>
-        <v>52.2915483690579</v>
+        <v>274.829413802094</v>
       </c>
       <c r="K8" s="13" t="n">
         <f aca="false">Financials!K12</f>
-        <v>124.399658705181</v>
+        <v>356.233844953188</v>
       </c>
       <c r="L8" s="13" t="n">
         <f aca="false">Financials!L12</f>
-        <v>185.152679307549</v>
+        <v>427.402552118134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7134,47 +7134,47 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">Financials!B18</f>
-        <v>-34.246</v>
+        <v>184.112</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">Financials!C18</f>
-        <v>-43.4453949901557</v>
+        <v>146.885314430029</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">Financials!D18</f>
-        <v>-141.466812363457</v>
+        <v>25.8251890540409</v>
       </c>
       <c r="E10" s="13" t="n">
         <f aca="false">Financials!E18</f>
-        <v>-131.481840248741</v>
+        <v>21.4649297760491</v>
       </c>
       <c r="F10" s="13" t="n">
         <f aca="false">Financials!F18</f>
-        <v>-170.563829178882</v>
+        <v>-36.1402489697512</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">Financials!G18</f>
-        <v>-121.850467213118</v>
+        <v>5.48585360402841</v>
       </c>
       <c r="H10" s="13" t="n">
         <f aca="false">Financials!H18</f>
-        <v>-68.0821056374046</v>
+        <v>52.5989671046498</v>
       </c>
       <c r="I10" s="13" t="n">
         <f aca="false">Financials!I18</f>
-        <v>-12.7471223809656</v>
+        <v>102.564736390111</v>
       </c>
       <c r="J10" s="13" t="n">
         <f aca="false">Financials!J18</f>
-        <v>25.5227901272649</v>
+        <v>134.140480977241</v>
       </c>
       <c r="K10" s="13" t="n">
         <f aca="false">Financials!K18</f>
-        <v>55.5108551213139</v>
+        <v>158.962215510334</v>
       </c>
       <c r="L10" s="13" t="n">
         <f aca="false">Financials!L18</f>
-        <v>75.5354482233106</v>
+        <v>174.364440562075</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7188,47 +7188,47 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">Dynamics!C9</f>
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">Dynamics!D9</f>
-        <v>434.1249</v>
+        <v>520.94988</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">Dynamics!E9</f>
-        <v>400.988146383</v>
+        <v>481.1857756596</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">Dynamics!F9</f>
-        <v>376.445089919586</v>
+        <v>451.734107903503</v>
       </c>
       <c r="F13" s="13" t="n">
         <f aca="false">Dynamics!G9</f>
-        <v>361.307637833258</v>
+        <v>432.050590086963</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">Dynamics!H9</f>
-        <v>356.50799079789</v>
+        <v>424.228608630819</v>
       </c>
       <c r="H13" s="13" t="n">
         <f aca="false">Dynamics!I9</f>
-        <v>356.586568252961</v>
+        <v>421.727141737555</v>
       </c>
       <c r="I13" s="13" t="n">
         <f aca="false">Dynamics!J9</f>
-        <v>362.880556354413</v>
+        <v>426.078162245627</v>
       </c>
       <c r="J13" s="13" t="n">
         <f aca="false">Dynamics!K9</f>
-        <v>368.724174704576</v>
+        <v>429.866141421397</v>
       </c>
       <c r="K13" s="13" t="n">
         <f aca="false">Dynamics!L9</f>
-        <v>373.293858346427</v>
+        <v>432.281031174332</v>
       </c>
       <c r="L13" s="13" t="n">
         <f aca="false">Dynamics!M9</f>
-        <v>375.089257845092</v>
+        <v>431.608799439813</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7237,47 +7237,47 @@
       </c>
       <c r="B14" s="13" t="n">
         <f aca="false">Dynamics!C20</f>
-        <v>180</v>
+        <v>216</v>
       </c>
       <c r="C14" s="13" t="n">
         <f aca="false">Dynamics!D20</f>
-        <v>189.0609</v>
+        <v>226.87308</v>
       </c>
       <c r="D14" s="13" t="n">
         <f aca="false">Dynamics!E20</f>
-        <v>197.0333124045</v>
+        <v>236.4399748854</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">Dynamics!F20</f>
-        <v>240.183750465257</v>
+        <v>286.433222381017</v>
       </c>
       <c r="F14" s="13" t="n">
         <f aca="false">Dynamics!G20</f>
-        <v>235.216515404029</v>
+        <v>278.849615202722</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">Dynamics!H20</f>
-        <v>296.535176377208</v>
+        <v>349.151636039641</v>
       </c>
       <c r="H14" s="13" t="n">
         <f aca="false">Dynamics!I20</f>
-        <v>346.03178740321</v>
+        <v>405.346275973246</v>
       </c>
       <c r="I14" s="13" t="n">
         <f aca="false">Dynamics!J20</f>
-        <v>391.842278850273</v>
+        <v>457.147893990672</v>
       </c>
       <c r="J14" s="13" t="n">
         <f aca="false">Dynamics!K20</f>
-        <v>417.355424646685</v>
+        <v>485.34664200267</v>
       </c>
       <c r="K14" s="13" t="n">
         <f aca="false">Dynamics!L20</f>
-        <v>433.946326589705</v>
+        <v>503.238613011294</v>
       </c>
       <c r="L14" s="13" t="n">
         <f aca="false">Dynamics!M20</f>
-        <v>442.592568495713</v>
+        <v>511.946747097495</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7384,47 +7384,47 @@
       </c>
       <c r="B17" s="13" t="n">
         <f aca="false">Dynamics!C53</f>
-        <v>140.4</v>
+        <v>161.46</v>
       </c>
       <c r="C17" s="13" t="n">
         <f aca="false">Dynamics!D53</f>
-        <v>139.61025</v>
+        <v>160.5517875</v>
       </c>
       <c r="D17" s="13" t="n">
         <f aca="false">Dynamics!E53</f>
-        <v>142.96449375</v>
+        <v>164.4091678125</v>
       </c>
       <c r="E17" s="13" t="n">
         <f aca="false">Dynamics!F53</f>
-        <v>153.031337803991</v>
+        <v>175.191155171178</v>
       </c>
       <c r="F17" s="13" t="n">
         <f aca="false">Dynamics!G53</f>
-        <v>163.435248747396</v>
+        <v>186.334248051888</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">Dynamics!H53</f>
-        <v>181.48166965732</v>
+        <v>206.044414848945</v>
       </c>
       <c r="H17" s="13" t="n">
         <f aca="false">Dynamics!I53</f>
-        <v>205.56342950497</v>
+        <v>232.620215179915</v>
       </c>
       <c r="I17" s="13" t="n">
         <f aca="false">Dynamics!J53</f>
-        <v>235.592635802739</v>
+        <v>265.930622115096</v>
       </c>
       <c r="J17" s="13" t="n">
         <f aca="false">Dynamics!K53</f>
-        <v>266.172129555558</v>
+        <v>299.896990765497</v>
       </c>
       <c r="K17" s="13" t="n">
         <f aca="false">Dynamics!L53</f>
-        <v>312.570067928302</v>
+        <v>351.697080819466</v>
       </c>
       <c r="L17" s="13" t="n">
         <f aca="false">Dynamics!M53</f>
-        <v>369.249979476113</v>
+        <v>415.028584558776</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7487,47 +7487,47 @@
       </c>
       <c r="B21" s="13" t="n">
         <f aca="false">Dynamics!C11</f>
-        <v>20.5</v>
+        <v>185</v>
       </c>
       <c r="C21" s="13" t="n">
         <f aca="false">Dynamics!D11</f>
-        <v>16.3404929755802</v>
+        <v>167.521544803419</v>
       </c>
       <c r="D21" s="13" t="n">
         <f aca="false">Dynamics!E11</f>
-        <v>9.39726420934655</v>
+        <v>148.576813869532</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">Dynamics!F11</f>
-        <v>4.22957758895538</v>
+        <v>134.62074480769</v>
       </c>
       <c r="F21" s="13" t="n">
         <f aca="false">Dynamics!G11</f>
-        <v>5.14288471075322</v>
+        <v>127.513146339018</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">Dynamics!H11</f>
-        <v>7.17208164607029</v>
+        <v>124.252565799909</v>
       </c>
       <c r="H21" s="13" t="n">
         <f aca="false">Dynamics!I11</f>
-        <v>13.080062113087</v>
+        <v>125.694136681189</v>
       </c>
       <c r="I21" s="13" t="n">
         <f aca="false">Dynamics!J11</f>
-        <v>22.3829536851132</v>
+        <v>131.674254165026</v>
       </c>
       <c r="J21" s="13" t="n">
         <f aca="false">Dynamics!K11</f>
-        <v>30.74461522519</v>
+        <v>136.547680673667</v>
       </c>
       <c r="K21" s="13" t="n">
         <f aca="false">Dynamics!L11</f>
-        <v>37.7814117319108</v>
+        <v>139.947839844731</v>
       </c>
       <c r="L21" s="13" t="n">
         <f aca="false">Dynamics!M11</f>
-        <v>43.0042223497528</v>
+        <v>141.009358443652</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7536,47 +7536,47 @@
       </c>
       <c r="B22" s="13" t="n">
         <f aca="false">Dynamics!C22</f>
-        <v>26.5</v>
+        <v>62.5</v>
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">Dynamics!D22</f>
-        <v>27.1158940499523</v>
+        <v>64.9280740499523</v>
       </c>
       <c r="D22" s="13" t="n">
         <f aca="false">Dynamics!E22</f>
-        <v>26.2456243040768</v>
+        <v>65.6522867849768</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">Dynamics!F22</f>
-        <v>41.1798841366883</v>
+        <v>87.4293560524479</v>
       </c>
       <c r="F22" s="13" t="n">
         <f aca="false">Dynamics!G22</f>
-        <v>41.7157579339878</v>
+        <v>85.3488577326803</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">Dynamics!H22</f>
-        <v>65.5792667770498</v>
+        <v>118.195726439483</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">Dynamics!I22</f>
-        <v>86.0755154745097</v>
+        <v>145.390004044546</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">Dynamics!J22</f>
-        <v>105.402737312138</v>
+        <v>170.708352452536</v>
       </c>
       <c r="J22" s="13" t="n">
         <f aca="false">Dynamics!K22</f>
-        <v>116.501440509386</v>
+        <v>184.492657865371</v>
       </c>
       <c r="K22" s="13" t="n">
         <f aca="false">Dynamics!L22</f>
-        <v>123.340527806587</v>
+        <v>192.632814228175</v>
       </c>
       <c r="L22" s="13" t="n">
         <f aca="false">Dynamics!M22</f>
-        <v>126.400638775888</v>
+        <v>195.75481737767</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7683,47 +7683,47 @@
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">Dynamics!C55</f>
-        <v>21.16</v>
+        <v>63.28</v>
       </c>
       <c r="C25" s="13" t="n">
         <f aca="false">Dynamics!D55</f>
-        <v>14.868305250031</v>
+        <v>57.1903289375232</v>
       </c>
       <c r="D25" s="13" t="n">
         <f aca="false">Dynamics!E55</f>
-        <v>11.2518629182462</v>
+        <v>55.0521946886847</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">Dynamics!F55</f>
-        <v>13.3207369263118</v>
+        <v>59.0682045129191</v>
       </c>
       <c r="F25" s="13" t="n">
         <f aca="false">Dynamics!G55</f>
-        <v>14.4501311130624</v>
+        <v>62.235409826138</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">Dynamics!H55</f>
-        <v>19.1480904239344</v>
+        <v>70.9642304239066</v>
       </c>
       <c r="H25" s="13" t="n">
         <f aca="false">Dynamics!I55</f>
-        <v>25.1942554229409</v>
+        <v>82.8933346183934</v>
       </c>
       <c r="I25" s="13" t="n">
         <f aca="false">Dynamics!J55</f>
-        <v>33.643952523837</v>
+        <v>99.0391096559203</v>
       </c>
       <c r="J25" s="13" t="n">
         <f aca="false">Dynamics!K55</f>
-        <v>41.2315259107779</v>
+        <v>114.701538031912</v>
       </c>
       <c r="K25" s="13" t="n">
         <f aca="false">Dynamics!L55</f>
-        <v>54.2088165283426</v>
+        <v>140.343642269497</v>
       </c>
       <c r="L25" s="13" t="n">
         <f aca="false">Dynamics!M55</f>
-        <v>70.3355572091107</v>
+        <v>172.142767858524</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="B47" s="13" t="n">
         <f aca="false">Financials!B22</f>
-        <v>2892.65888036717</v>
+        <v>6677.3529419064</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8402,7 +8402,7 @@
       </c>
       <c r="B48" s="20" t="n">
         <f aca="false">Financials!B25</f>
-        <v>-533.068478540835</v>
+        <v>786.151878438808</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="B49" s="20" t="n">
         <f aca="false">Financials!B26</f>
-        <v>647.029405555871</v>
+        <v>3510.26502278248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>